<commit_message>
Liste des questions et documents à transmettre par le FPPN ; PBC du 23/10/2026 sans doublon (90 items)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QrZoDwZJKb9thfUp96Ro9x
</commit_message>
<xml_diff>
--- a/FPPN_PBC_complete_pointee_20261023.xlsx
+++ b/FPPN_PBC_complete_pointee_20261023.xlsx
@@ -16,14 +16,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Points à clarifier" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pointage autres équipes" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pointage nouveaux fichiers" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pointage lot 1 (contenu)" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pointage lots 2 et 3 (contenu)" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pointage 22-10 (partie 1)" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pointage 22-10 (partie 2)" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pointage dossier compta 22-10" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'PBC Actuariat FPPN'!$B$12:$P$12</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'PBC Actuariat FPPN'!$1:$9</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'PBC Actuariat FPPN'!$A$1:$N$123</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'PBC Actuariat FPPN'!$A$1:$N$120</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Synthèse du pointage'!$5:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Synthèse du pointage'!$A$1:$D$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Détail par mois'!$B$5:$E$1605</definedName>
@@ -31,8 +31,8 @@
     <definedName name="_xlnm.Print_Area" localSheetId="6">'Points à clarifier'!$A$1:$F$66</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'Pointage autres équipes'!$5:$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="8">'Pointage nouveaux fichiers'!$5:$5</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="9">'Pointage lot 1 (contenu)'!$5:$5</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="10">'Pointage lots 2 et 3 (contenu)'!$5:$5</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="9">'Pointage 22-10 (partie 1)'!$5:$5</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="10">'Pointage 22-10 (partie 2)'!$5:$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="11">'Pointage dossier compta 22-10'!$5:$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -1036,7 +1036,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B4:M122"/>
+  <dimension ref="B4:M119"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.18359375" defaultRowHeight="13.5" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="4.82" customWidth="1" style="44" min="1" max="1"/>
@@ -1082,7 +1082,7 @@
     </row>
     <row r="7" ht="13.5" customHeight="1" s="48">
       <c r="M7" s="53">
-        <f>IFERROR(COUNTIF($M$11:$M$122,"Reçu")/(COUNTA($M$11:$M$122)-COUNTIF($M$11:$M$122,"Non Applicable")),0)</f>
+        <f>IFERROR(COUNTIF($M$11:$M$119,"Reçu")/(COUNTA($M$11:$M$119)-COUNTIF($M$11:$M$119,"Non Applicable")),0)</f>
         <v/>
       </c>
     </row>
@@ -1183,14 +1183,14 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="357" customHeight="1" s="48">
+    <row r="12" ht="417" customHeight="1" s="48">
       <c r="B12" s="70">
         <f>+B11+1</f>
         <v/>
       </c>
       <c r="C12" s="71" t="inlineStr">
         <is>
-          <t>Convention conclue avec la CGRAE pour la prise en charge des retraités, et ses avenants.</t>
+          <t>Convention conclue avec la CGRAE pour la prise en charge des retraités, ses avenants, son annexe 2 (bulletin de souscription), le barème de la cotisation des retraités et la liste des retraités souscripteurs non précomptés faute de quotité cessible suffisante.</t>
         </is>
       </c>
       <c r="E12" s="72" t="inlineStr">
@@ -1213,7 +1213,8 @@
           <t>Convention et avenants : non reçus. Reçu, fichiers de gestion : précomptes retour CGRAE : 30 mois sur 80 (février à mai 2024, juillet 2024 à août 2026) ; manque : janvier 2020 à janvier 2024, juin 2024. Bordereaux : 26 mois sur 80 (février 2024 à septembre 2025, novembre 2025 à janvier 2026, mai à juillet 2026) ; manque : janvier 2020 à janvier 2024, octobre 2025, février à avril 2026, août 2026. Pièces des retraités : 28 mois sur 80 (février 2024 à janvier 2026, mai à août 2026) ; manque : janvier 2020 à janvier 2024, février à avril 2026.
 Pointage des autres équipes (22/10/2026) : Tableau récapitulatif des contrats et conventions (dont CGRAE) reçu partiellement par l'équipe comptable ; liste complète en attente.
 Nouveaux fichiers du 22/10/2026 : Convention avec la CGRAE reçue ; avenants à vérifier. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « CONVENTION DE PARTENARIAT ENTRE IPS-CGRAE ET LE FPPN.pdf » (scan, 9 p.).
-Lots 2 et 3 lus le 22/10/2026 : Lu : « CONVENTION DE PARTENARIAT ENTRE IPS-CGRAE ET LE FPPN.pdf » (scan) : précompte sur pension des cotisations de prise en charge médicale (art. 3), pas de suspension des soins pour retard de la CGRAE (art. 4.1 e), précompte dans la limite de la quotité cessible (art. 4.2 a), aucun frais de gestion (art. 5). Annexe 2 (bulletin de souscription) et montant de la cotisation non reçus.</t>
+Lu le 22/10/2026 : Lu : « CONVENTION DE PARTENARIAT ENTRE IPS-CGRAE ET LE FPPN.pdf » (scan) : précompte sur pension des cotisations de prise en charge médicale (art. 3), pas de suspension des soins pour retard de la CGRAE (art. 4.1 e), précompte dans la limite de la quotité cessible (art. 4.2 a), aucun frais de gestion (art. 5). Annexe 2 (bulletin de souscription) et montant de la cotisation non reçus.
+Fusion du 23/10/2026 : reprend l'ancien item 114 (« Annexe 2 de la convention IPS-CGRAE (bulletin de souscription), barème de la cotisation des retraités et liste des retraités souscripteurs non précomptés faute … »), statut « Non Reçu ».</t>
         </is>
       </c>
       <c r="M12" s="76" t="inlineStr">
@@ -1259,8 +1260,8 @@
           <t>Non reçu dans l'envoi du 15/10/2026.
 Pointage des autres équipes (22/10/2026) : Rapports actuariels et calcul des provisions : en attente pour l'équipe comptable également.
 Nouveaux fichiers du 22/10/2026 : Études techniques internes reçues ; aucun rapport actuariel ni calcul des provisions. Contenu à analyser. Fichiers : 05-Nouveaux Prestations : « ETUDE DES RATIO MALADIE DECES 2.xlsx » ; « RAPPORT GLOBAL SUR LE SERVICE ASSURANCE MALADIE » (.docx, .pdf).
-Lot 1 lu le 22/10/2026 : Études internes reçues (« ETUDE DES RATIO MALADIE DECES 2.xlsx », « RAPPORT GLOBAL SUR LE SERVICE ASSURANCE MALADIE », « INTERPRETATION DES RATIOS… ») ; aucun rapport actuariel ni calcul des provisions.
-Lots 2 et 3 lus le 22/10/2026 : Lus : rapports de gestion et rapports moraux 2020 à 2025 (« RAPPORT DE GESTION 2020 FPPN - BASE - 10 (A).docx », « 1- RAPPORT MORAL 30 juin 2021 définitif (A).docx », « RAPPORT MORAL 2022 (définitif) (A).docx », « BILAN_DE_L'EXERCICE_CLOS_31.12.2023_(corrigé_et_finalisé)[1].pdf », « RAPPORT DE GESTION DETAILLE EXERCICE 2024.pdf », « RAPPORT GESTION NOUVEAUpdf.pdf », « Rapport de Gestion  2025 Final (2).pdf ») : analyses de l'excédent et de l'épargne, sans calcul actuariel des engagements.
+Lu le 22/10/2026 : Études internes reçues (« ETUDE DES RATIO MALADIE DECES 2.xlsx », « RAPPORT GLOBAL SUR LE SERVICE ASSURANCE MALADIE », « INTERPRETATION DES RATIOS… ») ; aucun rapport actuariel ni calcul des provisions.
+Lu le 22/10/2026 : Lus : rapports de gestion et rapports moraux 2020 à 2025 (« RAPPORT DE GESTION 2020 FPPN - BASE - 10 (A).docx », « 1- RAPPORT MORAL 30 juin 2021 définitif (A).docx », « RAPPORT MORAL 2022 (définitif) (A).docx », « BILAN_DE_L'EXERCICE_CLOS_31.12.2023_(corrigé_et_finalisé)[1].pdf », « RAPPORT DE GESTION DETAILLE EXERCICE 2024.pdf », « RAPPORT GESTION NOUVEAUpdf.pdf », « Rapport de Gestion  2025 Final (2).pdf ») : analyses de l'excédent et de l'épargne, sans calcul actuariel des engagements.
 Fusion du 23/10/2026 : reprend l'ancien item 48 (« Étude actuarielle des risques longs déposée à l'AIRMS, le cas échéant (règlement d'exécution n° 004/2022, art. 14). »), statut « Non Reçu ».</t>
         </is>
       </c>
@@ -1390,7 +1391,7 @@
         <is>
           <t>Reçu : fichiers aller (envoyés par le FPPN) et retour (précomptes de la Solde ou de la CGRAE), par mutualiste et par mois. Maladie 936 : 31 mois sur 80 (janvier à novembre 2024, janvier 2025 à août 2026) ; illisible : décembre 2024 ; manque : 2020 à 2023. Décès 8Z6 : 24 mois sur 80 (janvier à avril 2024, novembre 2024, janvier à mars 2025, mai 2025 à août 2026) ; illisible : décembre 2024 ; manque : 2020 à 2023, mai à octobre 2024, avril 2025. Retraités CGRAE : 30 mois sur 80 (février à mai 2024, juillet 2024 à août 2026) ; manque : janvier 2020 à janvier 2024, juin 2024. Manque : état des cotisations appelées et encaissées par mois et par catégorie.
 Pointage des autres équipes (22/10/2026) : Précomptes 2020 à 2022 (Easy Money) et état des cotisations de la Solde 2020 à 2023 non reçus ; aucun rapprochement entre fichiers retour et comptabilité (relance 2.2 : non applicable).
-Lots 2 et 3 lus le 22/10/2026 : Les rapports de gestion donnent les cotisations maladie annuelles (« Cotisation Maladie (3,5 % SB) »), sans détail mensuel ni par catégorie (« RAPPORT DE GESTION 2020 FPPN - BASE - 10 (A).docx », « 1- RAPPORT MORAL 30 juin 2021 définitif (A).docx », « RAPPORT MORAL 2022 (définitif) (A).docx », « BILAN_DE_L'EXERCICE_CLOS_31.12.2023_(corrigé_et_finalisé)[1].pdf », « RAPPORT DE GESTION DETAILLE EXERCICE 2024.pdf », « RAPPORT GESTION NOUVEAUpdf.pdf », « Rapport de Gestion  2025 Final (2).pdf »).</t>
+Lu le 22/10/2026 : Les rapports de gestion donnent les cotisations maladie annuelles (« Cotisation Maladie (3,5 % SB) »), sans détail mensuel ni par catégorie (« RAPPORT DE GESTION 2020 FPPN - BASE - 10 (A).docx », « 1- RAPPORT MORAL 30 juin 2021 définitif (A).docx », « RAPPORT MORAL 2022 (définitif) (A).docx », « BILAN_DE_L'EXERCICE_CLOS_31.12.2023_(corrigé_et_finalisé)[1].pdf », « RAPPORT DE GESTION DETAILLE EXERCICE 2024.pdf », « RAPPORT GESTION NOUVEAUpdf.pdf », « Rapport de Gestion  2025 Final (2).pdf »).</t>
         </is>
       </c>
       <c r="M18" s="76" t="inlineStr">
@@ -1645,7 +1646,7 @@
           <t>Non reçu dans l'envoi du 15/10/2026.
 Pointage des autres équipes (22/10/2026) : Dossiers des programmes immobiliers en attente (liste des immeubles : M. Koffi).
 Nouveaux fichiers du 22/10/2026 : Titres et baux reçus ; valeurs et dernières évaluations non reçues. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : certificats de propriété, acte de vente, « CONTRAT DE BAIL SONAPIE N° 2124-03002 / 03037 FPPN.pdf ».
-Lots 2 et 3 lus le 22/10/2026 : Titres de propriété du siège (Marcory) et du terrain du Plateau reçus ; inventaire et évaluation des biens non reçus.</t>
+Lu le 22/10/2026 : Titres de propriété du siège (Marcory) et du terrain du Plateau reçus ; inventaire et évaluation des biens non reçus.</t>
         </is>
       </c>
       <c r="M27" s="76" t="inlineStr">
@@ -1725,7 +1726,7 @@
           <t>Non reçu dans l'envoi du 15/10/2026.
 Pointage des autres équipes (22/10/2026) : Organigramme 2022 (identité et postes) reçu partiellement par l'équipe comptable ; version numérique en attente.
 Nouveaux fichiers du 22/10/2026 : Organigrammes 2020 et 2021 et un courrier de nomination reçus ; contacts des responsables non reçus. Contenu à analyser. Fichiers : « ORGANIGRAMME FPPN 2021(1).pdf » ; 03-Nouveaux Juridiques : « OrganigrammeFPPN_ORI (A) 2020.docx » ; « COURRIER DE NOMINATION DÉFINITIVE.pdf ».
-Lots 2 et 3 lus le 22/10/2026 : Lus : « OrganigrammeFPPN_ORI (A) 2020.docx », « ORGANIGRAMME FPPN 2021(1).pdf », « COURRIER DE NOMINATION DÉFINITIVE.pdf » ; contacts des responsables non reçus.</t>
+Lu le 22/10/2026 : Lus : « OrganigrammeFPPN_ORI (A) 2020.docx », « ORGANIGRAMME FPPN 2021(1).pdf », « COURRIER DE NOMINATION DÉFINITIVE.pdf » ; contacts des responsables non reçus.</t>
         </is>
       </c>
       <c r="M30" s="76" t="inlineStr">
@@ -1774,7 +1775,7 @@
         <is>
           <t>Non reçu dans l'envoi du 15/10/2026.
 Nouveaux fichiers du 22/10/2026 : Sinistralité observée par le FPPN (au 30 juin, historique 2015 à 2021) et interprétation : méthode du FPPN à confronter à la formule de la Décision n° 05/2022. Contenu à analyser. Fichiers : 05-Nouveaux Prestations : « ETUDE DES RATIO MALADIE DECES 2.xlsx » (onglets Tableau, Notes, Historique 2015-2021) ; « INTERPRETATION DES RATIOS… » (.docx, .pdf).
-Lot 1 lu le 22/10/2026 : Lu : « ETUDE DES RATIO MALADIE DECES 2.xlsx » : cotisations et sinistres décès, nombre d'adhérents et de décès (adhérents, conjoints, enfants) de 2015 au 30/06/2026 ; notes de calcul de la sinistralité décès (13 %) et maladie (99,23 %) au 30/06/2026. Détail mensuel maladie non reçu.</t>
+Lu le 22/10/2026 : Lu : « ETUDE DES RATIO MALADIE DECES 2.xlsx » : cotisations et sinistres décès, nombre d'adhérents et de décès (adhérents, conjoints, enfants) de 2015 au 30/06/2026 ; notes de calcul de la sinistralité décès (13 %) et maladie (99,23 %) au 30/06/2026. Détail mensuel maladie non reçu.</t>
         </is>
       </c>
       <c r="M32" s="76" t="inlineStr">
@@ -1855,7 +1856,7 @@
           <t>Non reçu dans l'envoi du 15/10/2026.
 Pointage des autres équipes (22/10/2026) : Barèmes en vigueur reçus dans la « cartographie des risques » (20/10/2026). Barèmes successifs depuis 2001 et décisions non reçus. Copie à obtenir auprès de l'équipe d'audit comptable.
 Nouveaux fichiers du 22/10/2026 : Barèmes 2021 reçus ; barèmes successifs depuis 2001 non reçus. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : cahiers des charges 2021 ; 05-Nouveaux Prestations : cartographie des risques.
-Lot 1 lu le 22/10/2026 : Barèmes 2021 à 2026 reçus (« CARTOGRAPHIE DES RISQUES COUVERTS ET DES PRESTATIONS OFFERTES.docx ») ; barèmes successifs de 2001 à 2020 et décisions non reçus.
+Lu le 22/10/2026 : Barèmes 2021 à 2026 reçus (« CARTOGRAPHIE DES RISQUES COUVERTS ET DES PRESTATIONS OFFERTES.docx ») ; barèmes successifs de 2001 à 2020 et décisions non reçus.
 Fusion du 23/10/2026 : reprend l'ancien item 93 (« Barème officiel des allocations décès par grade (sous-officier, officier, commissaire). »), statut « Reçu ».
 Fusion du 23/10/2026 : reprend l'ancien item 101 (« Tableau des allocations en vigueur de 2020 au 31/08/2026 : allocation décès du membre, allocation décès des ayants droit, allocation d'invalidité par corps (art… »), statut « Reçu ».
 Barème en vigueur lu dans « CARTOGRAPHIE DES RISQUES COUVERTS ET DES PRESTATIONS OFFERTES.docx » : officier 1 600 000 FCFA, sous-officier 1 400 000 FCFA.</t>
@@ -1970,7 +1971,7 @@
         <is>
           <t>Non reçu dans l'envoi du 15/10/2026.
 Pointage des autres équipes (22/10/2026) : Rapports de contrôle de l'AIRMS reçus en version papier par l'équipe comptable ; plan de redressement à rechercher. Copie à obtenir auprès de l'équipe d'audit comptable.
-Lots 2 et 3 lus le 22/10/2026 : Lus : « PLAN D'ACTION 2024.pdf » et « Plan d'action 2025.pdf » ; rapport de contrôle de l'AIRMS et plan de redressement non reçus.
+Lu le 22/10/2026 : Lus : « PLAN D'ACTION 2024.pdf » et « Plan d'action 2025.pdf » ; rapport de contrôle de l'AIRMS et plan de redressement non reçus.
 Fusion du 23/10/2026 : reprend l'ancien item 8 (« Correspondances avec l'AIRMS portant sur les réserves, les provisions ou les indicateurs prudentiels (observations, mises en demeure, plans de redressement). »), statut « Partiellement Reçu ».</t>
         </is>
       </c>
@@ -2238,7 +2239,7 @@
       <c r="J46" s="74" t="n"/>
       <c r="K46" s="75" t="inlineStr">
         <is>
-          <t>Demande issue de la lecture des textes de l'AIRMS (rapport v3, partie 10).
+          <t>Demande issue de la lecture des textes de l'AIRMS (rapport, partie 10).
 Pointage des autres équipes (22/10/2026) : Actes d'agrément et correspondances avec l'AIRMS reçus en version papier par l'équipe comptable ; version numérique en attente. Copie à obtenir auprès de l'équipe d'audit comptable.
 Nouveaux fichiers du 22/10/2026 : Attestation d'immatriculation n° 1D/0052016/CI du 05/04/2017 reçue ; décision d'agrément et liste des risques autorisés à vérifier. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « NUMERO D'IMMATRICULATION AIRSM N° 1D-0052016-CI DU 05-04-2017.pdf » (scan).</t>
         </is>
@@ -2276,10 +2277,10 @@
       <c r="J47" s="74" t="n"/>
       <c r="K47" s="75" t="inlineStr">
         <is>
-          <t>Demande issue de la lecture des textes de l'AIRMS (rapport v3, partie 10).
+          <t>Demande issue de la lecture des textes de l'AIRMS (rapport, partie 10).
 Pointage des autres équipes (22/10/2026) : États financiers reçus par l'équipe comptable. Rapports du commissaire aux comptes 2022 à 2025 en attente, 2020 et 2021 à retrouver par le FPPN.
 Nouveaux fichiers du 22/10/2026 : États financiers 2020 au 31/08/2026 reçus ; rapports du commissaire aux comptes et états par risque long non reçus. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « ETATS FINANCIERS 2020.pdf » à « ETATS FINANCIERS 2025.pdf », « ETATS FINANCIERS AU 31-08-2026.pdf » (scans) ; « BILAN_DE_L'EXERCICE_CLOS_31.12.2023_(corrigé_et_finalisé)[1].pdf ».
-Lots 2 et 3 lus le 22/10/2026 : Lus : « ETATS FINANCIERS 2020.pdf » à « ETATS FINANCIERS 2025.pdf » et « ETATS FINANCIERS AU 31-08-2026.pdf » (scans). Totaux de l'actif brut, résultat et trésorerie identiques aux balances, sauf 2023 (version antérieure : actif brut inférieur de 10 000 000 FCFA, excédent de 928 699 102 contre 930 629 102 FCFA) et résultat au 31/08/2026 (-437 148 460 contre -441 256 500 FCFA). Rapports du commissaire aux comptes et états par risque long non reçus.</t>
+Lu le 22/10/2026 : Lus : « ETATS FINANCIERS 2020.pdf » à « ETATS FINANCIERS 2025.pdf » et « ETATS FINANCIERS AU 31-08-2026.pdf » (scans). Totaux de l'actif brut, résultat et trésorerie identiques aux balances, sauf 2023 (version antérieure : actif brut inférieur de 10 000 000 FCFA, excédent de 928 699 102 contre 930 629 102 FCFA) et résultat au 31/08/2026 (-437 148 460 contre -441 256 500 FCFA). Rapports du commissaire aux comptes et états par risque long non reçus.</t>
         </is>
       </c>
       <c r="M47" s="76" t="inlineStr">
@@ -2313,7 +2314,7 @@
       <c r="J48" s="74" t="n"/>
       <c r="K48" s="75" t="inlineStr">
         <is>
-          <t>Demande issue de la lecture des textes de l'AIRMS (rapport v3, partie 10).</t>
+          <t>Demande issue de la lecture des textes de l'AIRMS (rapport, partie 10).</t>
         </is>
       </c>
       <c r="M48" s="76" t="inlineStr">
@@ -2347,7 +2348,7 @@
       <c r="J49" s="74" t="n"/>
       <c r="K49" s="75" t="inlineStr">
         <is>
-          <t>Demande issue de la lecture des textes de l'AIRMS (rapport v3, partie 10).</t>
+          <t>Demande issue de la lecture des textes de l'AIRMS (rapport, partie 10).</t>
         </is>
       </c>
       <c r="M49" s="76" t="inlineStr">
@@ -2356,7 +2357,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="477" customHeight="1" s="48">
+    <row r="50" ht="462" customHeight="1" s="48">
       <c r="B50" s="70">
         <f>+B49+1</f>
         <v/>
@@ -2383,10 +2384,10 @@
       <c r="J50" s="74" t="n"/>
       <c r="K50" s="75" t="inlineStr">
         <is>
-          <t>Demande issue de la lecture des textes de l'AIRMS (rapport v3, partie 10).
+          <t>Demande issue de la lecture des textes de l'AIRMS (rapport, partie 10).
 Pointage des autres équipes (22/10/2026) : Procès-verbaux des AG, CA et commissions reçus par l'équipe comptable, sauf 2020 et 2023. Copie à obtenir auprès de l'équipe d'audit comptable.
 Nouveaux fichiers du 22/10/2026 : PV de 2024 et compositions des organes reçus ; calendrier statutaire et autres PV à compléter. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « PV AG ORDINAIRE DU 15 FEVRIER 2024.pdf » ; listes des administrateurs et membres de la commission de surveillance.
-Lots 2 et 3 lus le 22/10/2026 : Lus : listes des administrateurs et des membres de la commission de surveillance et de contrôle d'août 2020 et d'août 2023 (scans) ; calendrier et PV des réunions non reçus.
+Lu le 22/10/2026 : Lus : listes des administrateurs et des membres de la commission de surveillance et de contrôle d'août 2020 et d'août 2023 (scans) ; calendrier et PV des réunions non reçus.
 Dossier « 08-Nouveaux Dossiers Compta » lu le 22/10/2026 : Lu : « ATTESTATION DE DESIGNATION DU DGFPPN AU TITRE DE LA MANDATURE 2020-2023.pdf » : directeur général désigné le 04/09/2020 pour la mandature 2020-2023 (AG du 27/08/2020) ; désignation après 2023 non reçue.
 Fusion du 23/10/2026 : reprend l'ancien item 5 (« Procès-verbaux ou décisions du Conseil d'administration et de l'Assemblée générale ayant modifié les cotisations, les prestations ou les taux servis sur l'éparg… »), statut « Non Reçu ».
 Fusion du 23/10/2026 : reprend l'ancien item 106 (« Procès-verbal de l'Assemblée Générale approuvant le reclassement des provisions techniques en comptes 15801000 et 15802000 en 2024 (article 75 des statuts). »), statut « Non Reçu ».
@@ -2424,7 +2425,7 @@
       <c r="J51" s="74" t="n"/>
       <c r="K51" s="75" t="inlineStr">
         <is>
-          <t>Demande issue de la lecture des textes de l'AIRMS (rapport v3, partie 10).
+          <t>Demande issue de la lecture des textes de l'AIRMS (rapport, partie 10).
 Fusion du 23/10/2026 : reprend l'ancien item 24 (« Politique de placement approuvée par le Conseil d'administration, si elle existe. »), statut « Non Reçu ».</t>
         </is>
       </c>
@@ -2461,8 +2462,8 @@
       <c r="J52" s="74" t="n"/>
       <c r="K52" s="75" t="inlineStr">
         <is>
-          <t>Demande issue de la lecture des textes de l'AIRMS (rapport v3, partie 10).
-Lots 2 et 3 lus le 22/10/2026 : Le rapport de gestion 2023 corrigé nomme la structure : Centre Médical du Policier (CMP). Statut juridique non reçu.
+          <t>Demande issue de la lecture des textes de l'AIRMS (rapport, partie 10).
+Lu le 22/10/2026 : Le rapport de gestion 2023 corrigé nomme la structure : Centre Médical du Policier (CMP). Statut juridique non reçu.
 Dossier « 08-Nouveaux Dossiers Compta » lu le 22/10/2026 : Lu : « ARRETE N° 0027-MSHP-DGS-DEPS DU 10-02-2020 PORTANT AUTORISATION D'OUVERTURE D'EXPLOITATION ET IMMATRICULATION DU CMP.pdf » : « Centre médical du FPPN », établissement sanitaire privé mutualiste, Yopougon Andokoi, immatriculé PV-ABIDJ-MEDIC/CMMU-02978-0022/2020, FPPN promoteur et propriétaire (art. 3). Comptabilité séparée non reçue (voir les nouveaux items).
 Sigle CMP : Clinique médicale du policier.</t>
         </is>
@@ -2480,7 +2481,7 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="162" customFormat="1" customHeight="1" s="68">
+    <row r="54" ht="222" customFormat="1" customHeight="1" s="68">
       <c r="B54" s="70">
         <f>+B52+1</f>
         <v/>
@@ -2513,7 +2514,8 @@
         <is>
           <t>Demande issue de l'entretien du 19/10/2026 avec le responsable des cotisations (PBC complémentaire cotisations).
 Fusion du 23/10/2026 : reprend l'ancien item 3 (« Barème des cotisations par catégorie de membres (actifs, retraités, autres) pour chaque année de 2020 à 2026, et répartition de la cotisation entre les garantie… »), statut « Partiellement Reçu ».
-Fusion du 23/10/2026 : reprend l'ancien item 45 (« Barème officiel des cotisations (décision, statuts ou règlement intérieur) fixant la répartition du taux de 5 % entre maladie et décès. »), statut « Reçu ».</t>
+Fusion du 23/10/2026 : reprend l'ancien item 45 (« Barème officiel des cotisations (décision, statuts ou règlement intérieur) fixant la répartition du taux de 5 % entre maladie et décès. »), statut « Reçu ».
+Fusion du 23/10/2026 : reprend l'ancien item 111 (« Clé de répartition maladie (936) / décès (8Z6) appliquée en janvier et février 2024 (rapport médian 8Z6 / 936 de 0,3059 et 0,3023, contre 0,3263 ensuite) et lis… »), statut « Non Reçu ».</t>
         </is>
       </c>
       <c r="M54" s="76" t="inlineStr">
@@ -2529,7 +2531,7 @@
       </c>
       <c r="C55" s="71" t="inlineStr">
         <is>
-          <t>Documentation de chaque produit : EFC, PEP, MEDOC, prêts du Grenier, flotte automobile (règlement, conditions de souscription, montants, conditions de sortie et de remboursement).</t>
+          <t>Documentation de chaque produit : EFC, PEP, prêts du Grenier, flotte automobile (règlement, conditions de souscription, montants, conditions de sortie et de remboursement). MEDOC est demandé à part.</t>
         </is>
       </c>
       <c r="E55" s="72" t="inlineStr">
@@ -2555,7 +2557,7 @@
         <is>
           <t>Demande issue de l'entretien du 19/10/2026 avec le responsable des cotisations (PBC complémentaire cotisations).
 Nouveaux fichiers du 22/10/2026 : EFC, PEP et Grenier documentés ; MEDOC et flotte automobile non documentés. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : manuel de produit d'épargne, cahiers des charges 2021, « POLITIK DE CREDIT DU GRENIER VFVF.doc ».
-Lot 1 lu le 22/10/2026 : EFC, PEP (« CAHIER DE CHARGEEFC &amp; PEP 2021.pdf », « MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx »), Grenier (« POLITIK DE CREDIT DU GRENIER VFVF.doc ») et flotte automobile (« MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx », chapitre II) documentés ; MEDOC non documenté.
+Lu le 22/10/2026 : EFC, PEP (« CAHIER DE CHARGEEFC &amp; PEP 2021.pdf », « MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx »), Grenier (« POLITIK DE CREDIT DU GRENIER VFVF.doc ») et flotte automobile (« MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx », chapitre II) documentés ; MEDOC non documenté.
 Fusion du 23/10/2026 : reprend l'ancien item 60 (« Date de démarrage (et, le cas échéant, de suspension) de chaque produit : EFC, PEP, MEDOC, prêts du Grenier, flotte automobile, cotisations des retraités (CGRAE… »), statut « Non Reçu ».</t>
         </is>
       </c>
@@ -2979,7 +2981,7 @@
     <row r="67" ht="18" customHeight="1" s="48">
       <c r="C67" s="69" t="inlineStr">
         <is>
-          <t>Provisions et engagements (revue du rapport v5, 19/10/2026)</t>
+          <t>Provisions et engagements (demande complémentaire du 19/10/2026)</t>
         </is>
       </c>
     </row>
@@ -3014,7 +3016,7 @@
       </c>
       <c r="K68" s="75" t="inlineStr">
         <is>
-          <t>Revue des provisions (rapport v5) : analyse en attente de ce document.
+          <t>Revue des provisions (rapport) : analyse en attente de ce document.
 Pointage des autres équipes (22/10/2026) : Décès et invalidité : états 2019 au 30/06/2026 reçus par l'équipe comptable (dates de survenance, déclaration et paiement à vérifier). Maladie : aucun suivi par dossier hors comptabilité, selon le FPPN. Copie à obtenir auprès de l'équipe d'audit comptable.
 Reformulée le 22/10/2026 : la méthode courte de provision demande, pour chaque facture, la date des soins, du dépôt et du paiement.
 Fusion du 23/10/2026 : reprend l'ancien item 13 (« Fichier des prestations payées du 01/01/2020 au 31/08/2026. Une ligne par dossier : matricule, type de prestation, date de l'événement (décès, soins, départ à l… »), statut « Partiellement Reçu ».
@@ -3054,7 +3056,7 @@
       <c r="J69" s="74" t="n"/>
       <c r="K69" s="75" t="inlineStr">
         <is>
-          <t>Revue des provisions (rapport v5) : analyse en attente de ce document.
+          <t>Revue des provisions (rapport) : analyse en attente de ce document.
 Dossier « 08-Nouveaux Dossiers Compta » lu le 22/10/2026 : Les états de fin d'année expliquent la dette du 41591000 ; aucune note ne fonde la provision obsèques (15802000) ni la provision maladie (15801000).
 Fusion du 23/10/2026 : reprend l'ancien item 6 (« Détail des provisions inscrites au bilan, par nature et par garantie, au 31/12/2019, 31/12/2020, 31/12/2021, 31/12/2022, 31/12/2023, 31/12/2024, 31/12/2025 et 3… »), statut « Partiellement Reçu ».
 Vérification du 23/10/2026 : montants identiques du report à nouveau du 01/09/2020 au 31/08/2026 ; seul mouvement, le reclassement de 2024 au même montant. Ce sont les provisions héritées décrites par le chef comptable.</t>
@@ -3097,7 +3099,7 @@
       </c>
       <c r="K70" s="75" t="inlineStr">
         <is>
-          <t>Revue des provisions (rapport v5) : analyse en attente de ce document.
+          <t>Revue des provisions (rapport) : analyse en attente de ce document.
 Pointage des autres équipes (22/10/2026) : Portefeuille des crédits reçu ; politique de dépréciation non tenue (« garanties et 1 % » selon le FPPN).</t>
         </is>
       </c>
@@ -3134,10 +3136,10 @@
       <c r="J71" s="74" t="n"/>
       <c r="K71" s="75" t="inlineStr">
         <is>
-          <t>Revue des provisions (rapport v5) : analyse en attente de ce document.
+          <t>Revue des provisions (rapport) : analyse en attente de ce document.
 Pointage des autres équipes (22/10/2026) : Règlement des crédits reçu ; aucune politique écrite de dépréciation (le FPPN cite les garanties et un taux de 1 %). Copie à obtenir auprès de l'équipe d'audit comptable.
 Nouveaux fichiers du 22/10/2026 : Politique de crédit du Grenier. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « POLITIK DE CREDIT DU GRENIER VFVF.doc ».
-Lot 1 lu le 22/10/2026 : Reçu : « POLITIK DE CREDIT DU GRENIER VFVF.doc » (environ 98 000 caractères) ; lecture détaillée à faire pour la dépréciation des prêts.</t>
+Lu le 22/10/2026 : Reçu : « POLITIK DE CREDIT DU GRENIER VFVF.doc » (environ 98 000 caractères) ; lecture détaillée à faire pour la dépréciation des prêts.</t>
         </is>
       </c>
       <c r="M71" s="76" t="inlineStr">
@@ -3175,7 +3177,7 @@
       </c>
       <c r="K72" s="75" t="inlineStr">
         <is>
-          <t>Revue des provisions (rapport v5) : analyse en attente de ce document.</t>
+          <t>Revue des provisions (rapport) : analyse en attente de ce document.</t>
         </is>
       </c>
       <c r="M72" s="76" t="inlineStr">
@@ -3184,19 +3186,19 @@
         </is>
       </c>
     </row>
-    <row r="73" ht="132" customHeight="1" s="48">
+    <row r="73" ht="162" customHeight="1" s="48">
       <c r="B73" s="70">
         <f>+B72+1</f>
         <v/>
       </c>
       <c r="C73" s="71" t="inlineStr">
         <is>
-          <t>Note de calcul de la provision pour indemnités de départ à la retraite (compte 196) : méthode, hypothèses, liste des salariés.</t>
+          <t>Règles de la garantie santé des retraités : durée (à vie ou limitée), conditions, cotisation, décision qui la fonde.</t>
         </is>
       </c>
       <c r="E73" s="72" t="inlineStr">
         <is>
-          <t>Moyen</t>
+          <t>Urgent</t>
         </is>
       </c>
       <c r="G73" s="73" t="n">
@@ -3205,117 +3207,119 @@
       <c r="H73" s="73" t="n">
         <v>46321</v>
       </c>
-      <c r="I73" s="73" t="n"/>
+      <c r="I73" s="73" t="n">
+        <v>46317</v>
+      </c>
       <c r="J73" s="74" t="n"/>
       <c r="K73" s="75" t="inlineStr">
         <is>
-          <t>Revue des provisions (rapport v5) : analyse en attente de ce document.
-Pointage des autres équipes (22/10/2026) : Rapport actuariel et extraction de la provision pour départ à la retraite en attente (M. Koffi).
-Fusion du 23/10/2026 : reprend l'ancien item 98 (« Fichiers de calcul de la provision pour départ à la retraite de 2020 à 2026 (complète l'item 78). »), statut « Non Reçu ».</t>
+          <t>Revue des provisions (rapport) : analyse en attente de ce document.
+Lu le 22/10/2026 : La convention IPS-CGRAE confirme la garantie santé des retraités souscripteurs ; durée, cotisation et ayants droit couverts non précisés (« CONVENTION DE PARTENARIAT ENTRE IPS-CGRAE ET LE FPPN.pdf »).
+Fusion du 23/10/2026 : reprend l'ancien item 108 (« Décision fixant la situation des policiers retraités : maintien de la qualité de membre (article 7 des statuts), restitution de la carte (article 38 du règlemen… »), statut « Partiellement Reçu ».</t>
         </is>
       </c>
       <c r="M73" s="76" t="inlineStr">
         <is>
-          <t>Non Reçu</t>
-        </is>
-      </c>
-    </row>
-    <row r="74" ht="162" customHeight="1" s="48">
-      <c r="B74" s="70">
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="18" customHeight="1" s="48">
+      <c r="C74" s="69" t="inlineStr">
+        <is>
+          <t>Placements et autres actifs (entretiens du 19/10/2026, 14h)</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="177" customHeight="1" s="48">
+      <c r="B75" s="70">
         <f>+B73+1</f>
         <v/>
       </c>
-      <c r="C74" s="71" t="inlineStr">
-        <is>
-          <t>Règles de la garantie santé des retraités : durée (à vie ou limitée), conditions, cotisation, décision qui la fonde.</t>
-        </is>
-      </c>
-      <c r="E74" s="72" t="inlineStr">
+      <c r="C75" s="71" t="inlineStr">
+        <is>
+          <t>DAT BOA (comptes 52210200 et 52210300) : conventions, taux, échéances et relevés de 2020 au 31/08/2026, et réponse écrite à la question : le DAT du compte 52210200 est-il un placement du FPPN ou un placement affecté à l'EFC, comme l'indique l'intitulé du compte ?</t>
+        </is>
+      </c>
+      <c r="E75" s="72" t="inlineStr">
         <is>
           <t>Urgent</t>
         </is>
       </c>
-      <c r="G74" s="73" t="n">
+      <c r="G75" s="73" t="n">
         <v>46314</v>
       </c>
-      <c r="H74" s="73" t="n">
+      <c r="H75" s="73" t="n">
         <v>46321</v>
       </c>
-      <c r="I74" s="73" t="n">
+      <c r="I75" s="73" t="n">
         <v>46317</v>
       </c>
-      <c r="J74" s="74" t="n"/>
-      <c r="K74" s="75" t="inlineStr">
-        <is>
-          <t>Revue des provisions (rapport v5) : analyse en attente de ce document.
-Lots 2 et 3 lus le 22/10/2026 : La convention IPS-CGRAE confirme la garantie santé des retraités souscripteurs ; durée, cotisation et ayants droit couverts non précisés (« CONVENTION DE PARTENARIAT ENTRE IPS-CGRAE ET LE FPPN.pdf »).
-Fusion du 23/10/2026 : reprend l'ancien item 108 (« Décision fixant la situation des policiers retraités : maintien de la qualité de membre (article 7 des statuts), restitution de la carte (article 38 du règlemen… »), statut « Partiellement Reçu ».</t>
-        </is>
-      </c>
-      <c r="M74" s="76" t="inlineStr">
-        <is>
-          <t>Partiellement Reçu</t>
-        </is>
-      </c>
-    </row>
-    <row r="75" ht="18" customHeight="1" s="48">
-      <c r="C75" s="69" t="inlineStr">
-        <is>
-          <t>Placements et autres actifs (entretiens du 19/10/2026, 14h)</t>
-        </is>
-      </c>
-    </row>
-    <row r="76" ht="177" customHeight="1" s="48">
-      <c r="B76" s="70">
-        <f>+B74+1</f>
-        <v/>
-      </c>
-      <c r="C76" s="71" t="inlineStr">
-        <is>
-          <t>DAT BOA (comptes 52210200 et 52210300) : conventions, taux, échéances et relevés de 2020 au 31/08/2026, et réponse écrite à la question : le DAT du compte 52210200 est-il un placement du FPPN ou un placement affecté à l'EFC, comme l'indique l'intitulé du compte ?</t>
-        </is>
-      </c>
-      <c r="E76" s="72" t="inlineStr">
-        <is>
-          <t>Urgent</t>
-        </is>
-      </c>
-      <c r="G76" s="73" t="n">
-        <v>46314</v>
-      </c>
-      <c r="H76" s="73" t="n">
-        <v>46321</v>
-      </c>
-      <c r="I76" s="73" t="n">
-        <v>46317</v>
-      </c>
-      <c r="J76" s="74" t="inlineStr">
+      <c r="J75" s="74" t="inlineStr">
         <is>
           <t>Electronique</t>
         </is>
       </c>
-      <c r="K76" s="75" t="inlineStr">
+      <c r="K75" s="75" t="inlineStr">
         <is>
           <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).
 Pointage des autres équipes (22/10/2026) : Dossiers des DAT en attente pour l'équipe comptable également.
 Nouveaux fichiers du 22/10/2026 : Mouvements des comptes BOA à lire ; conventions et relevés du DAT non reçus. Contenu à analyser. Fichiers : 07-Nouveaux Trésorerie et placements : états de rapprochement bancaire 2020 à 2026.
-Lot 1 lu le 22/10/2026 : Mouvements mensuels des comptes BOA lisibles dans « ETAT DE RAPPROCHEMENT BANCAIRE FPPN 2020.xlsx » à « … 2026.xlsx » ; conventions, taux et relevés du DAT non reçus.</t>
+Lu le 22/10/2026 : Mouvements mensuels des comptes BOA lisibles dans « ETAT DE RAPPROCHEMENT BANCAIRE FPPN 2020.xlsx » à « … 2026.xlsx » ; conventions, taux et relevés du DAT non reçus.</t>
+        </is>
+      </c>
+      <c r="M75" s="76" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="42" customHeight="1" s="48">
+      <c r="B76" s="70">
+        <f>+B75+1</f>
+        <v/>
+      </c>
+      <c r="C76" s="71" t="inlineStr">
+        <is>
+          <t>Bulletin de souscription au FCP géré par United Capital (SGI), valeurs liquidatives et relevés de 2025 au 31/08/2026.</t>
+        </is>
+      </c>
+      <c r="E76" s="72" t="inlineStr">
+        <is>
+          <t>Urgent</t>
+        </is>
+      </c>
+      <c r="G76" s="73" t="n">
+        <v>46314</v>
+      </c>
+      <c r="H76" s="73" t="n">
+        <v>46321</v>
+      </c>
+      <c r="I76" s="73" t="n"/>
+      <c r="J76" s="74" t="inlineStr">
+        <is>
+          <t>Electronique</t>
+        </is>
+      </c>
+      <c r="K76" s="75" t="inlineStr">
+        <is>
+          <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).</t>
         </is>
       </c>
       <c r="M76" s="76" t="inlineStr">
         <is>
-          <t>Partiellement Reçu</t>
-        </is>
-      </c>
-    </row>
-    <row r="77" ht="42" customHeight="1" s="48">
+          <t>Non Reçu</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="132" customHeight="1" s="48">
       <c r="B77" s="70">
         <f>+B76+1</f>
         <v/>
       </c>
       <c r="C77" s="71" t="inlineStr">
         <is>
-          <t>Bulletin de souscription au FCP géré par United Capital (SGI), valeurs liquidatives et relevés de 2025 au 31/08/2026.</t>
+          <t>Inventaire et tableau de variation de tous les placements de 2016 au 31/08/2026 : souscriptions, intérêts, débouclages, par banque ou gestionnaire.</t>
         </is>
       </c>
       <c r="E77" s="72" t="inlineStr">
@@ -3329,7 +3333,9 @@
       <c r="H77" s="73" t="n">
         <v>46321</v>
       </c>
-      <c r="I77" s="73" t="n"/>
+      <c r="I77" s="73" t="n">
+        <v>46317</v>
+      </c>
       <c r="J77" s="74" t="inlineStr">
         <is>
           <t>Electronique</t>
@@ -3337,28 +3343,30 @@
       </c>
       <c r="K77" s="75" t="inlineStr">
         <is>
-          <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).</t>
+          <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).
+Pointage des autres équipes (22/10/2026) : Tableau de synthèse des placements en attente pour l'équipe comptable également.
+Fusion du 23/10/2026 : reprend l'ancien item 20 (« Échéancier des placements au 31/12/2025 et au 31/08/2026 : nature, établissement, montant, date de souscription, date d'échéance, taux, conditions de sortie ant… »), statut « Partiellement Reçu ».</t>
         </is>
       </c>
       <c r="M77" s="76" t="inlineStr">
         <is>
-          <t>Non Reçu</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" ht="132" customHeight="1" s="48">
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="102" customHeight="1" s="48">
       <c r="B78" s="70">
         <f>+B77+1</f>
         <v/>
       </c>
       <c r="C78" s="71" t="inlineStr">
         <is>
-          <t>Inventaire et tableau de variation de tous les placements de 2016 au 31/08/2026 : souscriptions, intérêts, débouclages, par banque ou gestionnaire.</t>
+          <t>Correspondance avec Orabank sur l'arrêt des prélèvements mensuels et le remboursement du DAT.</t>
         </is>
       </c>
       <c r="E78" s="72" t="inlineStr">
         <is>
-          <t>Urgent</t>
+          <t>Moyen</t>
         </is>
       </c>
       <c r="G78" s="73" t="n">
@@ -3370,16 +3378,11 @@
       <c r="I78" s="73" t="n">
         <v>46317</v>
       </c>
-      <c r="J78" s="74" t="inlineStr">
-        <is>
-          <t>Electronique</t>
-        </is>
-      </c>
+      <c r="J78" s="74" t="n"/>
       <c r="K78" s="75" t="inlineStr">
         <is>
           <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).
-Pointage des autres équipes (22/10/2026) : Tableau de synthèse des placements en attente pour l'équipe comptable également.
-Fusion du 23/10/2026 : reprend l'ancien item 20 (« Échéancier des placements au 31/12/2025 et au 31/08/2026 : nature, établissement, montant, date de souscription, date d'échéance, taux, conditions de sortie ant… »), statut « Partiellement Reçu ».</t>
+Nouveaux fichiers du 22/10/2026 : La convention doit préciser la dénomination et le statut de la structure CMP. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « CONVENTION TRANSVIE-CMP.pdf ».</t>
         </is>
       </c>
       <c r="M78" s="76" t="inlineStr">
@@ -3388,14 +3391,14 @@
         </is>
       </c>
     </row>
-    <row r="79" ht="102" customHeight="1" s="48">
+    <row r="79" ht="312" customHeight="1" s="48">
       <c r="B79" s="70">
         <f>+B78+1</f>
         <v/>
       </c>
       <c r="C79" s="71" t="inlineStr">
         <is>
-          <t>Correspondance avec Orabank sur l'arrêt des prélèvements mensuels et le remboursement du DAT.</t>
+          <t>Titres de propriété ou actes d'acquisition des terrains, situation de chaque terrain (projet, attribution, litige).</t>
         </is>
       </c>
       <c r="E79" s="72" t="inlineStr">
@@ -3416,7 +3419,10 @@
       <c r="K79" s="75" t="inlineStr">
         <is>
           <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).
-Nouveaux fichiers du 22/10/2026 : La convention doit préciser la dénomination et le statut de la structure CMP. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « CONVENTION TRANSVIE-CMP.pdf ».</t>
+Pointage des autres équipes (22/10/2026) : Titres de propriété et tableau de synthèse des biens en attente (M. Sangaré).
+Nouveaux fichiers du 22/10/2026 : Deux certificats de propriété et un acte de vente reçus ; situation de chaque terrain (projet, attribution, litige) non reçue. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « Certificat de Propriété Terrain Marcori (Siège).pdf » ; « Certificat de Propriété Terrain Plateau.pdf » ; « Vente ferme par les consorts SIRANSY TOURE SOULEYMANE… ».
+Lu le 22/10/2026 : Lus : « Certificat de Propriété Terrain Marcori (Siège).pdf », « Certificat de Propriété Terrain Plateau.pdf » et « Vente ferme par les consorts SIRANSY TOURE SOULEYMANE AU PROFIT DU FPPN.pdf » (lot n° 40 de 1 469 m²). Scans partiellement lisibles ; situation et valeur de chaque terrain non reçues.
+Dossier « 08-Nouveaux Dossiers Compta » lu le 22/10/2026 : Lu : « DEROGATION AUX REGLES D'URBANISME CONSTRUCTION 4 IMMEUBLES R+5 AVEC 01 CES DE 70% A USAGE D'HABITATION COCODY 2 PLTX.pdf » : accord de janvier 2025 pour quatre immeubles R+5 sur les lots 3005 à 3007, îlot 83, TF n° 119 230, Cocody. Budget et financement non reçus.</t>
         </is>
       </c>
       <c r="M79" s="76" t="inlineStr">
@@ -3425,19 +3431,19 @@
         </is>
       </c>
     </row>
-    <row r="80" ht="312" customHeight="1" s="48">
+    <row r="80" ht="102" customHeight="1" s="48">
       <c r="B80" s="70">
         <f>+B79+1</f>
         <v/>
       </c>
       <c r="C80" s="71" t="inlineStr">
         <is>
-          <t>Titres de propriété ou actes d'acquisition des terrains, situation de chaque terrain (projet, attribution, litige).</t>
+          <t>Baux et encaissements des immeubles d'Aboisso.</t>
         </is>
       </c>
       <c r="E80" s="72" t="inlineStr">
         <is>
-          <t>Moyen</t>
+          <t>Faible</t>
         </is>
       </c>
       <c r="G80" s="73" t="n">
@@ -3453,10 +3459,7 @@
       <c r="K80" s="75" t="inlineStr">
         <is>
           <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).
-Pointage des autres équipes (22/10/2026) : Titres de propriété et tableau de synthèse des biens en attente (M. Sangaré).
-Nouveaux fichiers du 22/10/2026 : Deux certificats de propriété et un acte de vente reçus ; situation de chaque terrain (projet, attribution, litige) non reçue. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « Certificat de Propriété Terrain Marcori (Siège).pdf » ; « Certificat de Propriété Terrain Plateau.pdf » ; « Vente ferme par les consorts SIRANSY TOURE SOULEYMANE… ».
-Lots 2 et 3 lus le 22/10/2026 : Lus : « Certificat de Propriété Terrain Marcori (Siège).pdf », « Certificat de Propriété Terrain Plateau.pdf » et « Vente ferme par les consorts SIRANSY TOURE SOULEYMANE AU PROFIT DU FPPN.pdf » (lot n° 40 de 1 469 m²). Scans partiellement lisibles ; situation et valeur de chaque terrain non reçues.
-Dossier « 08-Nouveaux Dossiers Compta » lu le 22/10/2026 : Lu : « DEROGATION AUX REGLES D'URBANISME CONSTRUCTION 4 IMMEUBLES R+5 AVEC 01 CES DE 70% A USAGE D'HABITATION COCODY 2 PLTX.pdf » : accord de janvier 2025 pour quatre immeubles R+5 sur les lots 3005 à 3007, îlot 83, TF n° 119 230, Cocody. Budget et financement non reçus.</t>
+Lu le 22/10/2026 : Lus : « CONTRAT DE BAIL SONAPIE N° 2124-03002 FPPN.pdf » et « … 2124-03037 FPPN.pdf » (scans peu lisibles, bail de deux ans, loyer trimestriel) ; objet à rapprocher des immeubles d'Aboisso, encaissements non reçus.</t>
         </is>
       </c>
       <c r="M80" s="76" t="inlineStr">
@@ -3465,19 +3468,19 @@
         </is>
       </c>
     </row>
-    <row r="81" ht="102" customHeight="1" s="48">
+    <row r="81" ht="87" customHeight="1" s="48">
       <c r="B81" s="70">
         <f>+B80+1</f>
         <v/>
       </c>
       <c r="C81" s="71" t="inlineStr">
         <is>
-          <t>Baux et encaissements des immeubles d'Aboisso.</t>
+          <t>Rapport de réévaluation du siège et décision de comptabilisation au compte 10620000.</t>
         </is>
       </c>
       <c r="E81" s="72" t="inlineStr">
         <is>
-          <t>Faible</t>
+          <t>Urgent</t>
         </is>
       </c>
       <c r="G81" s="73" t="n">
@@ -3487,13 +3490,13 @@
         <v>46321</v>
       </c>
       <c r="I81" s="73" t="n">
-        <v>46317</v>
+        <v>46316</v>
       </c>
       <c r="J81" s="74" t="n"/>
       <c r="K81" s="75" t="inlineStr">
         <is>
           <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).
-Lots 2 et 3 lus le 22/10/2026 : Lus : « CONTRAT DE BAIL SONAPIE N° 2124-03002 FPPN.pdf » et « … 2124-03037 FPPN.pdf » (scans peu lisibles, bail de deux ans, loyer trimestriel) ; objet à rapprocher des immeubles d'Aboisso, encaissements non reçus.</t>
+Fusion du 23/10/2026 : reprend l'ancien item 50 (« PV d'AG d'affectation des excédents 2023 à 2025 et origine du compte 10620000 « Réserve disponible ». »), statut « Partiellement Reçu ».</t>
         </is>
       </c>
       <c r="M81" s="76" t="inlineStr">
@@ -3502,19 +3505,19 @@
         </is>
       </c>
     </row>
-    <row r="82" ht="87" customHeight="1" s="48">
+    <row r="82" ht="42" customHeight="1" s="48">
       <c r="B82" s="70">
         <f>+B81+1</f>
         <v/>
       </c>
       <c r="C82" s="71" t="inlineStr">
         <is>
-          <t>Rapport de réévaluation du siège et décision de comptabilisation au compte 10620000.</t>
+          <t>Dossier de la créance sur l'hôpital de la Police (compte 47111100) : pièces, correspondances avec l'État, décision d'autonomie de l'hôpital.</t>
         </is>
       </c>
       <c r="E82" s="72" t="inlineStr">
         <is>
-          <t>Urgent</t>
+          <t>Moyen</t>
         </is>
       </c>
       <c r="G82" s="73" t="n">
@@ -3523,30 +3526,27 @@
       <c r="H82" s="73" t="n">
         <v>46321</v>
       </c>
-      <c r="I82" s="73" t="n">
-        <v>46316</v>
-      </c>
+      <c r="I82" s="73" t="n"/>
       <c r="J82" s="74" t="n"/>
       <c r="K82" s="75" t="inlineStr">
         <is>
-          <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).
-Fusion du 23/10/2026 : reprend l'ancien item 50 (« PV d'AG d'affectation des excédents 2023 à 2025 et origine du compte 10620000 « Réserve disponible ». »), statut « Partiellement Reçu ».</t>
+          <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).</t>
         </is>
       </c>
       <c r="M82" s="76" t="inlineStr">
         <is>
-          <t>Partiellement Reçu</t>
-        </is>
-      </c>
-    </row>
-    <row r="83" ht="42" customHeight="1" s="48">
+          <t>Non Reçu</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="207" customHeight="1" s="48">
       <c r="B83" s="70">
         <f>+B82+1</f>
         <v/>
       </c>
       <c r="C83" s="71" t="inlineStr">
         <is>
-          <t>Dossier de la créance sur l'hôpital de la Police (compte 47111100) : pièces, correspondances avec l'État, décision d'autonomie de l'hôpital.</t>
+          <t>Convention d'apporteur d'affaires avec GNA et décomptes annuels des commissions (20 % des primes collectées).</t>
         </is>
       </c>
       <c r="E83" s="72" t="inlineStr">
@@ -3560,45 +3560,11 @@
       <c r="H83" s="73" t="n">
         <v>46321</v>
       </c>
-      <c r="I83" s="73" t="n"/>
+      <c r="I83" s="73" t="n">
+        <v>46310</v>
+      </c>
       <c r="J83" s="74" t="n"/>
       <c r="K83" s="75" t="inlineStr">
-        <is>
-          <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).</t>
-        </is>
-      </c>
-      <c r="M83" s="76" t="inlineStr">
-        <is>
-          <t>Non Reçu</t>
-        </is>
-      </c>
-    </row>
-    <row r="84" ht="207" customHeight="1" s="48">
-      <c r="B84" s="70">
-        <f>+B83+1</f>
-        <v/>
-      </c>
-      <c r="C84" s="71" t="inlineStr">
-        <is>
-          <t>Convention d'apporteur d'affaires avec GNA et décomptes annuels des commissions (20 % des primes collectées).</t>
-        </is>
-      </c>
-      <c r="E84" s="72" t="inlineStr">
-        <is>
-          <t>Moyen</t>
-        </is>
-      </c>
-      <c r="G84" s="73" t="n">
-        <v>46314</v>
-      </c>
-      <c r="H84" s="73" t="n">
-        <v>46321</v>
-      </c>
-      <c r="I84" s="73" t="n">
-        <v>46310</v>
-      </c>
-      <c r="J84" s="74" t="n"/>
-      <c r="K84" s="75" t="inlineStr">
         <is>
           <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).
 Pointage des autres équipes (22/10/2026) : Tableau récapitulatif des conventions (dont GNA) reçu partiellement par l'équipe comptable ; liste complète en attente.
@@ -3606,25 +3572,67 @@
 Fusion du 23/10/2026 : reprend l'ancien item 68 (« États de GNA sur la flotte automobile : primes reçues, soldes par adhérent, trop-perçus remboursés, de 2020 à août 2026, et convention avec GNA. »), statut « Non Reçu ».</t>
         </is>
       </c>
+      <c r="M83" s="76" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="162" customHeight="1" s="48">
+      <c r="B84" s="70">
+        <f>+B83+1</f>
+        <v/>
+      </c>
+      <c r="C84" s="71" t="inlineStr">
+        <is>
+          <t>Liste des comptes bancaires, actifs et inactifs, avec leurs signataires.</t>
+        </is>
+      </c>
+      <c r="E84" s="72" t="inlineStr">
+        <is>
+          <t>Moyen</t>
+        </is>
+      </c>
+      <c r="G84" s="73" t="n">
+        <v>46314</v>
+      </c>
+      <c r="H84" s="73" t="n">
+        <v>46321</v>
+      </c>
+      <c r="I84" s="73" t="n">
+        <v>46317</v>
+      </c>
+      <c r="J84" s="74" t="inlineStr">
+        <is>
+          <t>Electronique</t>
+        </is>
+      </c>
+      <c r="K84" s="75" t="inlineStr">
+        <is>
+          <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).
+Pointage des autres équipes (22/10/2026) : Liste des comptes bancaires reçue partiellement par l'équipe comptable ; liste par exercice en attente. Copie à obtenir auprès de l'équipe d'audit comptable.
+Nouveaux fichiers du 22/10/2026 : Liste des comptes bancaires et habilitations de signature. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « LISTE DES COMPTES BANCAIRES  DU FPPN.pdf » ; « Habilitation de signatures.pdf » (scans).</t>
+        </is>
+      </c>
       <c r="M84" s="76" t="inlineStr">
         <is>
-          <t>Partiellement Reçu</t>
-        </is>
-      </c>
-    </row>
-    <row r="85" ht="162" customHeight="1" s="48">
+          <t>Reçu</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="102" customHeight="1" s="48">
       <c r="B85" s="70">
         <f>+B84+1</f>
         <v/>
       </c>
       <c r="C85" s="71" t="inlineStr">
         <is>
-          <t>Liste des comptes bancaires, actifs et inactifs, avec leurs signataires.</t>
+          <t>État des chèques en suspens et des chèques annulés lors des changements de signataires.</t>
         </is>
       </c>
       <c r="E85" s="72" t="inlineStr">
         <is>
-          <t>Moyen</t>
+          <t>Faible</t>
         </is>
       </c>
       <c r="G85" s="73" t="n">
@@ -3644,114 +3652,107 @@
       <c r="K85" s="75" t="inlineStr">
         <is>
           <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).
-Pointage des autres équipes (22/10/2026) : Liste des comptes bancaires reçue partiellement par l'équipe comptable ; liste par exercice en attente. Copie à obtenir auprès de l'équipe d'audit comptable.
-Nouveaux fichiers du 22/10/2026 : Liste des comptes bancaires et habilitations de signature. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « LISTE DES COMPTES BANCAIRES  DU FPPN.pdf » ; « Habilitation de signatures.pdf » (scans).</t>
+Lu le 22/10/2026 : Les rapprochements bancaires listent des chèques en suspens, dont certains émis depuis décembre 2021 sur le compte BOA EFC et encore non débités au 31/12/2025 (« ETAT DE RAPPROCHEMENT BANCAIRE FPPN 2020.xlsx » à « … 2026.xlsx »).</t>
         </is>
       </c>
       <c r="M85" s="76" t="inlineStr">
         <is>
-          <t>Reçu</t>
-        </is>
-      </c>
-    </row>
-    <row r="86" ht="102" customHeight="1" s="48">
-      <c r="B86" s="70">
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="18" customHeight="1" s="48">
+      <c r="C86" s="69" t="inlineStr">
+        <is>
+          <t>Provisions (entretiens du 19/10/2026, 16h)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="222" customHeight="1" s="48">
+      <c r="B87" s="70">
         <f>+B85+1</f>
         <v/>
       </c>
-      <c r="C86" s="71" t="inlineStr">
-        <is>
-          <t>État des chèques en suspens et des chèques annulés lors des changements de signataires.</t>
-        </is>
-      </c>
-      <c r="E86" s="72" t="inlineStr">
-        <is>
-          <t>Faible</t>
-        </is>
-      </c>
-      <c r="G86" s="73" t="n">
+      <c r="C87" s="71" t="inlineStr">
+        <is>
+          <t>Fichiers des décès transmis par la direction du personnel et calcul de fin d'année des allocations restant à payer, de 2020 à 2025, avec le compte utilisé.</t>
+        </is>
+      </c>
+      <c r="E87" s="72" t="inlineStr">
+        <is>
+          <t>Urgent</t>
+        </is>
+      </c>
+      <c r="G87" s="73" t="n">
         <v>46314</v>
       </c>
-      <c r="H86" s="73" t="n">
+      <c r="H87" s="73" t="n">
         <v>46321</v>
       </c>
-      <c r="I86" s="73" t="n">
+      <c r="I87" s="73" t="n">
         <v>46317</v>
       </c>
-      <c r="J86" s="74" t="inlineStr">
+      <c r="J87" s="74" t="inlineStr">
         <is>
           <t>Electronique</t>
         </is>
       </c>
-      <c r="K86" s="75" t="inlineStr">
-        <is>
-          <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).
-Lot 1 lu le 22/10/2026 : Les rapprochements bancaires listent des chèques en suspens, dont certains émis depuis décembre 2021 sur le compte BOA EFC et encore non débités au 31/12/2025 (« ETAT DE RAPPROCHEMENT BANCAIRE FPPN 2020.xlsx » à « … 2026.xlsx »).</t>
-        </is>
-      </c>
-      <c r="M86" s="76" t="inlineStr">
-        <is>
-          <t>Partiellement Reçu</t>
-        </is>
-      </c>
-    </row>
-    <row r="87" ht="18" customHeight="1" s="48">
-      <c r="C87" s="69" t="inlineStr">
-        <is>
-          <t>Provisions (entretiens du 19/10/2026, 16h)</t>
-        </is>
-      </c>
-    </row>
-    <row r="88" ht="222" customHeight="1" s="48">
-      <c r="B88" s="70">
-        <f>+B86+1</f>
-        <v/>
-      </c>
-      <c r="C88" s="71" t="inlineStr">
-        <is>
-          <t>Fichiers des décès transmis par la direction du personnel et calcul de fin d'année des allocations restant à payer, de 2020 à 2025, avec le compte utilisé.</t>
-        </is>
-      </c>
-      <c r="E88" s="72" t="inlineStr">
-        <is>
-          <t>Urgent</t>
-        </is>
-      </c>
-      <c r="G88" s="73" t="n">
-        <v>46314</v>
-      </c>
-      <c r="H88" s="73" t="n">
-        <v>46321</v>
-      </c>
-      <c r="I88" s="73" t="n">
-        <v>46317</v>
-      </c>
-      <c r="J88" s="74" t="inlineStr">
-        <is>
-          <t>Electronique</t>
-        </is>
-      </c>
-      <c r="K88" s="75" t="inlineStr">
+      <c r="K87" s="75" t="inlineStr">
         <is>
           <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).
 Dossier « 08-Nouveaux Dossiers Compta » lu le 22/10/2026 : Reçus : « PROV ALLOCATION DECES 2021.xlsx », « PROV ALLOCATION DECES 2022.xlsx », « ALLOC DECES 2023 PAYER ET A PROVISIONNER .xlsx », « PROV ALLOCATION DECES 2024.xlsx », « PROV ALLOCATIONS DECES ET FRAIS FUNERAIRES 2025.xlsx ». Calcul de fin d'année au barème, comptabilisé au compte 41591000 (au franc près en 2024 et 2025). Fichiers des décès transmis par la direction du personnel non reçus ; écarts 2021 à 2023 à expliquer.
 Vérification du 23/10/2026 : le calcul de fin d'année est comptabilisé au compte 41591000 (2024 : 140 800 000 FCFA ; 2025 : 130 600 000 FCFA, égal au crédit de l'année). Point résolu sur le compte utilisé.</t>
         </is>
       </c>
+      <c r="M87" s="76" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="102" customHeight="1" s="48">
+      <c r="B88" s="70">
+        <f>+B87+1</f>
+        <v/>
+      </c>
+      <c r="C88" s="71" t="inlineStr">
+        <is>
+          <t>Contrats et décomptes de gestion de la garantie décès avec LMAI et Sanlam.</t>
+        </is>
+      </c>
+      <c r="E88" s="72" t="inlineStr">
+        <is>
+          <t>Moyen</t>
+        </is>
+      </c>
+      <c r="G88" s="73" t="n">
+        <v>46314</v>
+      </c>
+      <c r="H88" s="73" t="n">
+        <v>46321</v>
+      </c>
+      <c r="I88" s="73" t="n"/>
+      <c r="J88" s="74" t="n"/>
+      <c r="K88" s="75" t="inlineStr">
+        <is>
+          <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).
+Fusion du 23/10/2026 : reprend l'ancien item 32 (« Contrats conclus avec les assureurs pour la gestion externalisée (novembre 2013 à 2020), avec les primes payées et les sinistres réglés par année. »), statut « Non Reçu ».</t>
+        </is>
+      </c>
       <c r="M88" s="76" t="inlineStr">
         <is>
-          <t>Partiellement Reçu</t>
-        </is>
-      </c>
-    </row>
-    <row r="89" ht="102" customHeight="1" s="48">
+          <t>Non Reçu</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="87" customHeight="1" s="48">
       <c r="B89" s="70">
         <f>+B88+1</f>
         <v/>
       </c>
       <c r="C89" s="71" t="inlineStr">
         <is>
-          <t>Contrats et décomptes de gestion de la garantie décès avec LMAI et Sanlam.</t>
+          <t>Courrier de l'AIRMS demandant le reclassement des provisions en compte 158.</t>
         </is>
       </c>
       <c r="E89" s="72" t="inlineStr">
@@ -3770,7 +3771,7 @@
       <c r="K89" s="75" t="inlineStr">
         <is>
           <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).
-Fusion du 23/10/2026 : reprend l'ancien item 32 (« Contrats conclus avec les assureurs pour la gestion externalisée (novembre 2013 à 2020), avec les primes payées et les sinistres réglés par année. »), statut « Non Reçu ».</t>
+Pointage des autres équipes (22/10/2026) : À rechercher dans les correspondances avec l'AIRMS reçues en version papier par l'équipe comptable.</t>
         </is>
       </c>
       <c r="M89" s="76" t="inlineStr">
@@ -3779,14 +3780,14 @@
         </is>
       </c>
     </row>
-    <row r="90" ht="87" customHeight="1" s="48">
+    <row r="90" ht="42" customHeight="1" s="48">
       <c r="B90" s="70">
         <f>+B89+1</f>
         <v/>
       </c>
       <c r="C90" s="71" t="inlineStr">
         <is>
-          <t>Courrier de l'AIRMS demandant le reclassement des provisions en compte 158.</t>
+          <t>Notification du taux de risques professionnels (2 %) par la CNPS.</t>
         </is>
       </c>
       <c r="E90" s="72" t="inlineStr">
@@ -3804,8 +3805,7 @@
       <c r="J90" s="74" t="n"/>
       <c r="K90" s="75" t="inlineStr">
         <is>
-          <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).
-Pointage des autres équipes (22/10/2026) : À rechercher dans les correspondances avec l'AIRMS reçues en version papier par l'équipe comptable.</t>
+          <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).</t>
         </is>
       </c>
       <c r="M90" s="76" t="inlineStr">
@@ -3814,14 +3814,14 @@
         </is>
       </c>
     </row>
-    <row r="91" ht="42" customHeight="1" s="48">
+    <row r="91" ht="252" customHeight="1" s="48">
       <c r="B91" s="70">
         <f>+B90+1</f>
         <v/>
       </c>
       <c r="C91" s="71" t="inlineStr">
         <is>
-          <t>Notification du taux de risques professionnels (2 %) par la CNPS.</t>
+          <t>Déclarations CNPS de 2020 au 31/08/2026.</t>
         </is>
       </c>
       <c r="E91" s="72" t="inlineStr">
@@ -3835,32 +3835,42 @@
       <c r="H91" s="73" t="n">
         <v>46321</v>
       </c>
-      <c r="I91" s="73" t="n"/>
-      <c r="J91" s="74" t="n"/>
+      <c r="I91" s="73" t="n">
+        <v>46316</v>
+      </c>
+      <c r="J91" s="74" t="inlineStr">
+        <is>
+          <t>Electronique</t>
+        </is>
+      </c>
       <c r="K91" s="75" t="inlineStr">
         <is>
-          <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).</t>
+          <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).
+Pointage des autres équipes (22/10/2026) : DISA et état 301 reçus sauf 2026 ; ITS et FDFP reçus (2021 manquant) ; déclarations CNPS en attente. Copie à obtenir auprès de l'équipe d'audit comptable.
+Nouveaux fichiers du 22/10/2026 : DISA, état 301 et appels CNPS annuels reçus pour 2020 à 2025 ; déclarations mensuelles CNPS et 2026 non reçues. Contenu à analyser. Fichiers : 04-Nouveaux Personnel et paie : « ETAT 301 &amp; DISA 2020 à 2025 FPPN.xls », « DISA_256927_2021 à 2025.xls », DASC 2022, 2023, 2025.
+Lu le 22/10/2026 : Lu : états 301 et DISA 2020 à 2025, appels CNPS annuels, DASC 2022, 2023, 2025, fichiers e-CNPS complémentaires 2022. Déclarations mensuelles CNPS et 2026 non reçues.
+Lu le 22/10/2026 : DISA et DASC 2021 à 2025 scannées et états des travailleurs occasionnels 2024 et 2025, en double des fichiers Excel reçus.</t>
         </is>
       </c>
       <c r="M91" s="76" t="inlineStr">
         <is>
-          <t>Non Reçu</t>
-        </is>
-      </c>
-    </row>
-    <row r="92" ht="252" customHeight="1" s="48">
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="192" customHeight="1" s="48">
       <c r="B92" s="70">
         <f>+B91+1</f>
         <v/>
       </c>
       <c r="C92" s="71" t="inlineStr">
         <is>
-          <t>Déclarations CNPS de 2020 au 31/08/2026.</t>
+          <t>Décision fixant le taux servi de 3,5 % sur le PEP et l'EFC.</t>
         </is>
       </c>
       <c r="E92" s="72" t="inlineStr">
         <is>
-          <t>Moyen</t>
+          <t>Urgent</t>
         </is>
       </c>
       <c r="G92" s="73" t="n">
@@ -3870,20 +3880,15 @@
         <v>46321</v>
       </c>
       <c r="I92" s="73" t="n">
-        <v>46316</v>
-      </c>
-      <c r="J92" s="74" t="inlineStr">
-        <is>
-          <t>Electronique</t>
-        </is>
-      </c>
+        <v>46317</v>
+      </c>
+      <c r="J92" s="74" t="n"/>
       <c r="K92" s="75" t="inlineStr">
         <is>
           <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).
-Pointage des autres équipes (22/10/2026) : DISA et état 301 reçus sauf 2026 ; ITS et FDFP reçus (2021 manquant) ; déclarations CNPS en attente. Copie à obtenir auprès de l'équipe d'audit comptable.
-Nouveaux fichiers du 22/10/2026 : DISA, état 301 et appels CNPS annuels reçus pour 2020 à 2025 ; déclarations mensuelles CNPS et 2026 non reçues. Contenu à analyser. Fichiers : 04-Nouveaux Personnel et paie : « ETAT 301 &amp; DISA 2020 à 2025 FPPN.xls », « DISA_256927_2021 à 2025.xls », DASC 2022, 2023, 2025.
-Lot 1 lu le 22/10/2026 : Lu : états 301 et DISA 2020 à 2025, appels CNPS annuels, DASC 2022, 2023, 2025, fichiers e-CNPS complémentaires 2022. Déclarations mensuelles CNPS et 2026 non reçues.
-Lots 2 et 3 lus le 22/10/2026 : Lot 3 : DISA et DASC 2021 à 2025 scannées et états des travailleurs occasionnels 2024 et 2025, en double des fichiers Excel du lot 1.</t>
+Nouveaux fichiers du 22/10/2026 : Taux servi de 3,5 % à vérifier dans ces documents ; décision non reçue. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : manuel de produit d'épargne ; cahier des charges EFC et PEP 2021.
+Lu le 22/10/2026 : Le taux de 3,5 % n'est écrit que pour le PEP (« MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx ») ; pour l'EFC, les textes donnent 5,5 % ou 14 % simple. Décision non reçue.
+Fusion du 23/10/2026 : reprend l'ancien item 18 (« Taux d'intérêt crédité sur l'épargne chaque année et décision qui l'a fixé. »), statut « Partiellement Reçu ».</t>
         </is>
       </c>
       <c r="M92" s="76" t="inlineStr">
@@ -3892,60 +3897,65 @@
         </is>
       </c>
     </row>
-    <row r="93" ht="192" customHeight="1" s="48">
-      <c r="B93" s="70">
+    <row r="93" ht="18" customHeight="1" s="48">
+      <c r="C93" s="69" t="inlineStr">
+        <is>
+          <t>Textes du FPPN cités par les statuts et le règlement intérieur (lecture des textes du 15/06/2023)</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="327" customHeight="1" s="48">
+      <c r="B94" s="70">
         <f>+B92+1</f>
         <v/>
       </c>
-      <c r="C93" s="71" t="inlineStr">
-        <is>
-          <t>Décision fixant le taux servi de 3,5 % sur le PEP et l'EFC.</t>
-        </is>
-      </c>
-      <c r="E93" s="72" t="inlineStr">
+      <c r="C94" s="71" t="inlineStr">
+        <is>
+          <t>Cahier des charges du régime des prestations sociales du FPPN en vigueur, et versions applicables depuis 2020 (cité aux articles 21 et 40 à 42 du règlement intérieur).</t>
+        </is>
+      </c>
+      <c r="E94" s="72" t="inlineStr">
         <is>
           <t>Urgent</t>
         </is>
       </c>
-      <c r="G93" s="73" t="n">
+      <c r="G94" s="73" t="n">
         <v>46314</v>
       </c>
-      <c r="H93" s="73" t="n">
+      <c r="H94" s="73" t="n">
         <v>46321</v>
       </c>
-      <c r="I93" s="73" t="n">
+      <c r="I94" s="73" t="n">
         <v>46317</v>
       </c>
-      <c r="J93" s="74" t="n"/>
-      <c r="K93" s="75" t="inlineStr">
-        <is>
-          <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).
-Nouveaux fichiers du 22/10/2026 : Taux servi de 3,5 % à vérifier dans ces documents ; décision non reçue. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : manuel de produit d'épargne ; cahier des charges EFC et PEP 2021.
-Lot 1 lu le 22/10/2026 : Le taux de 3,5 % n'est écrit que pour le PEP (« MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx ») ; pour l'EFC, les textes donnent 5,5 % ou 14 % simple. Décision non reçue.
-Fusion du 23/10/2026 : reprend l'ancien item 18 (« Taux d'intérêt crédité sur l'épargne chaque année et décision qui l'a fixé. »), statut « Partiellement Reçu ».</t>
-        </is>
-      </c>
-      <c r="M93" s="76" t="inlineStr">
-        <is>
-          <t>Partiellement Reçu</t>
-        </is>
-      </c>
-    </row>
-    <row r="94" ht="18" customHeight="1" s="48">
-      <c r="C94" s="69" t="inlineStr">
-        <is>
-          <t>Textes du FPPN cités par les statuts et le règlement intérieur (lecture des textes du 15/06/2023)</t>
-        </is>
-      </c>
-    </row>
-    <row r="95" ht="327" customHeight="1" s="48">
+      <c r="J94" s="74" t="inlineStr">
+        <is>
+          <t>Physique et Electronique</t>
+        </is>
+      </c>
+      <c r="K94" s="75" t="inlineStr">
+        <is>
+          <t>Demande issue de la lecture des statuts et du règlement intérieur du 15/06/2023 (PBC complémentaire textes et personnel).
+Nouveaux fichiers du 22/10/2026 : Cahiers des charges du régime des prestations sociales, version 2021. Versions antérieures à 2021 non reçues. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « CAHIER DE CHARGE  MALADIES ET INVAL-DECES 2021.pdf » (17 p.) ; « CAHIER DE CHARGEEFC &amp; PEP 2021.pdf » (10 p.).
+Lu le 22/10/2026 : Lu : cahiers des charges 2021 « CAHIER DE CHARGE  MALADIES ET INVAL-DECES 2021.pdf » (risques couverts, ticket modérateur 80 % / 20 %, exclusions, forclusions, procédures) et « CAHIER DE CHARGEEFC &amp; PEP 2021.pdf ». Le tableau des allocations n'y figure pas (renvoi) : il est dans « CARTOGRAPHIE DES RISQUES COUVERTS ET DES PRESTATIONS OFFERTES.docx ». Versions antérieures à 2021 non reçues.
+Fusion du 23/10/2026 : reprend l'ancien item 2 (« Règlement ou fiche descriptive de chaque prestation servie (allocation décès, invalidité, prise en charge des retraités, santé, épargne, autres aides) : bénéfic… »), statut « Reçu ».
+Fusion du 23/10/2026 : reprend l'ancien item 33 (« Liste des pièces exigées pour chaque prestation et cahier du régime des prestations sociales. »), statut « Reçu ».</t>
+        </is>
+      </c>
+      <c r="M94" s="76" t="inlineStr">
+        <is>
+          <t>Reçu</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="297" customHeight="1" s="48">
       <c r="B95" s="70">
-        <f>+B93+1</f>
+        <f>+B94+1</f>
         <v/>
       </c>
       <c r="C95" s="71" t="inlineStr">
         <is>
-          <t>Cahier des charges du régime des prestations sociales du FPPN en vigueur, et versions applicables depuis 2020 (cité aux articles 21 et 40 à 42 du règlement intérieur).</t>
+          <t>Manuels de procédure du Plan Epargne Plus et de l'Entraide de Fin de Carrière : prestations, rémunération servie, conditions de sortie et de rachat (articles 69 et 71 du règlement intérieur).</t>
         </is>
       </c>
       <c r="E95" s="72" t="inlineStr">
@@ -3964,176 +3974,167 @@
       </c>
       <c r="J95" s="74" t="inlineStr">
         <is>
-          <t>Physique et Electronique</t>
+          <t>Electronique</t>
         </is>
       </c>
       <c r="K95" s="75" t="inlineStr">
-        <is>
-          <t>Demande issue de la lecture des statuts et du règlement intérieur du 15/06/2023 (PBC complémentaire textes et personnel).
-Nouveaux fichiers du 22/10/2026 : Cahiers des charges du régime des prestations sociales, version 2021. Versions antérieures à 2021 non reçues. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « CAHIER DE CHARGE  MALADIES ET INVAL-DECES 2021.pdf » (17 p.) ; « CAHIER DE CHARGEEFC &amp; PEP 2021.pdf » (10 p.).
-Lot 1 lu le 22/10/2026 : Lu : cahiers des charges 2021 « CAHIER DE CHARGE  MALADIES ET INVAL-DECES 2021.pdf » (risques couverts, ticket modérateur 80 % / 20 %, exclusions, forclusions, procédures) et « CAHIER DE CHARGEEFC &amp; PEP 2021.pdf ». Le tableau des allocations n'y figure pas (renvoi) : il est dans « CARTOGRAPHIE DES RISQUES COUVERTS ET DES PRESTATIONS OFFERTES.docx ». Versions antérieures à 2021 non reçues.
-Fusion du 23/10/2026 : reprend l'ancien item 2 (« Règlement ou fiche descriptive de chaque prestation servie (allocation décès, invalidité, prise en charge des retraités, santé, épargne, autres aides) : bénéfic… »), statut « Reçu ».
-Fusion du 23/10/2026 : reprend l'ancien item 33 (« Liste des pièces exigées pour chaque prestation et cahier du régime des prestations sociales. »), statut « Reçu ».</t>
-        </is>
-      </c>
-      <c r="M95" s="76" t="inlineStr">
-        <is>
-          <t>Reçu</t>
-        </is>
-      </c>
-    </row>
-    <row r="96" ht="297" customHeight="1" s="48">
-      <c r="B96" s="70">
-        <f>+B95+1</f>
-        <v/>
-      </c>
-      <c r="C96" s="71" t="inlineStr">
-        <is>
-          <t>Manuels de procédure du Plan Epargne Plus et de l'Entraide de Fin de Carrière : prestations, rémunération servie, conditions de sortie et de rachat (articles 69 et 71 du règlement intérieur).</t>
-        </is>
-      </c>
-      <c r="E96" s="72" t="inlineStr">
-        <is>
-          <t>Urgent</t>
-        </is>
-      </c>
-      <c r="G96" s="73" t="n">
-        <v>46314</v>
-      </c>
-      <c r="H96" s="73" t="n">
-        <v>46321</v>
-      </c>
-      <c r="I96" s="73" t="n">
-        <v>46317</v>
-      </c>
-      <c r="J96" s="74" t="inlineStr">
-        <is>
-          <t>Electronique</t>
-        </is>
-      </c>
-      <c r="K96" s="75" t="inlineStr">
         <is>
           <t>Demande issue de la lecture des statuts et du règlement intérieur du 15/06/2023 (PBC complémentaire textes et personnel).
 Pointage des autres équipes (22/10/2026) : À rechercher dans les manuels de procédures non signés reçus par l'équipe comptable le 21/10/2026.
 Nouveaux fichiers du 22/10/2026 : Manuel des produits d'épargne (PEP et EFC). Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx ».
-Lot 1 lu le 22/10/2026 : Lu : « MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx » (version 2021, certificat d'adoption non daté ni signé) : PEP rémunéré à 3,5 % par an, EFC à 5,5 % par an, intérêts non capitalisés et versés sur le compte courant.
+Lu le 22/10/2026 : Lu : « MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx » (version 2021, certificat d'adoption non daté ni signé) : PEP rémunéré à 3,5 % par an, EFC à 5,5 % par an, intérêts non capitalisés et versés sur le compte courant.
 Fusion du 23/10/2026 : reprend l'ancien item 16 (« Description des produits d'épargne (épargne de fin de carrière, Plan Épargne Plus, autres) : règles de versement, taux d'intérêt servi ou garanti, conditions de… »), statut « Reçu ».
 Fusion du 23/10/2026 : reprend l'ancien item 46 (« Règlement des produits PEP et EFC : conditions de retrait, échéances, âge de versement, taux servi. »), statut « Reçu ».</t>
         </is>
       </c>
-      <c r="M96" s="76" t="inlineStr">
-        <is>
-          <t>Reçu</t>
-        </is>
-      </c>
-    </row>
-    <row r="97" ht="18" customHeight="1" s="48">
-      <c r="C97" s="69" t="inlineStr">
+      <c r="M95" s="76" t="inlineStr">
+        <is>
+          <t>Reçu</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="18" customHeight="1" s="48">
+      <c r="C96" s="69" t="inlineStr">
         <is>
           <t>Personnel de la Direction Générale (périmètre de la provision pour départ à la retraite) (lecture des textes du 15/06/2023)</t>
         </is>
       </c>
     </row>
-    <row r="98" ht="357" customHeight="1" s="48">
-      <c r="B98" s="70">
-        <f>+B96+1</f>
+    <row r="97" ht="342" customHeight="1" s="48">
+      <c r="B97" s="70">
+        <f>+B95+1</f>
         <v/>
       </c>
-      <c r="C98" s="71" t="inlineStr">
-        <is>
-          <t>Fichier du personnel de la Direction Générale avec une colonne de statut : personnel civil salarié ou fonctionnaire de police en service (article 31 du règlement intérieur ; complète l'item 76).</t>
-        </is>
-      </c>
-      <c r="E98" s="72" t="inlineStr">
+      <c r="C97" s="71" t="inlineStr">
+        <is>
+          <t>Fichier du personnel de la Direction Générale au 31/12/2025 et au 31/08/2026 : date de naissance, date d'embauche, salaire mensuel, catégorie, statut (personnel civil salarié ou fonctionnaire de police en service, article 31 du règlement intérieur).</t>
+        </is>
+      </c>
+      <c r="E97" s="72" t="inlineStr">
         <is>
           <t>Urgent</t>
         </is>
       </c>
-      <c r="G98" s="73" t="n">
+      <c r="G97" s="73" t="n">
         <v>46314</v>
       </c>
-      <c r="H98" s="73" t="n">
+      <c r="H97" s="73" t="n">
         <v>46321</v>
       </c>
-      <c r="I98" s="73" t="n">
+      <c r="I97" s="73" t="n">
         <v>46317</v>
       </c>
-      <c r="J98" s="74" t="inlineStr">
+      <c r="J97" s="74" t="inlineStr">
         <is>
           <t>Electronique</t>
         </is>
       </c>
-      <c r="K98" s="75" t="inlineStr">
+      <c r="K97" s="75" t="inlineStr">
         <is>
           <t>Demande issue de la lecture des statuts et du règlement intérieur du 15/06/2023 (PBC complémentaire textes et personnel).
 Pointage des autres équipes (22/10/2026) : Mouvements du personnel et livres de paie en attente (M. Koffi) : le statut civil ou policier devra y figurer.
 Nouveaux fichiers du 22/10/2026 : Les DISA couvrent les salariés déclarés à la CNPS (personnel civil) ; les fonctionnaires de police en service n'y figurent a priori pas. Statut à confirmer. Contenu à analyser. Fichiers : 04-Nouveaux Personnel et paie : DISA 2021 à 2025 ; « RECAPSALAIRES » des états 301.
-Lot 1 lu le 22/10/2026 : Les DISA couvrent les salariés déclarés à la CNPS. Les états 301 distinguent des onglets « RECAPSALAIRES 2024 CMP » et « RECAPSALAIRES 2025 GRENIER » : Direction Générale, clinique et Grenier sont identifiables par nom. Le statut des policiers en service n'y figure pas.
-Lots 2 et 3 lus le 22/10/2026 : Organigrammes reçus ; le statut civil ou policier de chaque agent n'y figure pas. Rattachement aux entités établi par les récapitulatifs de salaires 2024 (CMP) et 2025 (Grenier).
+Lu le 22/10/2026 : Les DISA couvrent les salariés déclarés à la CNPS. Les états 301 distinguent des onglets « RECAPSALAIRES 2024 CMP » et « RECAPSALAIRES 2025 GRENIER » : Direction Générale, clinique et Grenier sont identifiables par nom. Le statut des policiers en service n'y figure pas.
+Lu le 22/10/2026 : Organigrammes reçus ; le statut civil ou policier de chaque agent n'y figure pas. Rattachement aux entités établi par les récapitulatifs de salaires 2024 (CMP) et 2025 (Grenier).
 Fusion du 23/10/2026 : reprend l'ancien item 76 (« Fichier du personnel du FPPN au 31/12/2025 et au 31/08/2026 : date de naissance, date d'embauche, salaire mensuel, catégorie, âge de départ prévu. »), statut « Partiellement Reçu ».</t>
         </is>
       </c>
+      <c r="M97" s="76" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="102" customHeight="1" s="48">
+      <c r="B98" s="70">
+        <f>+B97+1</f>
+        <v/>
+      </c>
+      <c r="C98" s="71" t="inlineStr">
+        <is>
+          <t>Contrat de travail type du personnel civil, convention collective appliquée et tout accord ou avenant fixant l'âge de départ et l'indemnité de départ à la retraite.</t>
+        </is>
+      </c>
+      <c r="E98" s="72" t="inlineStr">
+        <is>
+          <t>Moyen</t>
+        </is>
+      </c>
+      <c r="G98" s="73" t="n">
+        <v>46314</v>
+      </c>
+      <c r="H98" s="73" t="n">
+        <v>46321</v>
+      </c>
+      <c r="I98" s="73" t="n"/>
+      <c r="J98" s="74" t="n"/>
+      <c r="K98" s="75" t="inlineStr">
+        <is>
+          <t>Demande issue de la lecture des statuts et du règlement intérieur du 15/06/2023 (PBC complémentaire textes et personnel).
+Fusion du 23/10/2026 : reprend l'ancien item 77 (« Convention collective et accord d'entreprise applicables au personnel du FPPN, articles fixant l'indemnité de départ à la retraite. »), statut « Non Reçu ».</t>
+        </is>
+      </c>
       <c r="M98" s="76" t="inlineStr">
         <is>
-          <t>Partiellement Reçu</t>
-        </is>
-      </c>
-    </row>
-    <row r="99" ht="102" customHeight="1" s="48">
-      <c r="B99" s="70">
+          <t>Non Reçu</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="18" customHeight="1" s="48">
+      <c r="C99" s="69" t="inlineStr">
+        <is>
+          <t>Décisions des organes (lecture des textes du 15/06/2023)</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="72" customHeight="1" s="48">
+      <c r="B100" s="70">
         <f>+B98+1</f>
         <v/>
       </c>
-      <c r="C99" s="71" t="inlineStr">
-        <is>
-          <t>Contrat de travail type du personnel civil, convention collective appliquée et tout avenant fixant l'âge de départ à la retraite (complète l'item 77).</t>
-        </is>
-      </c>
-      <c r="E99" s="72" t="inlineStr">
-        <is>
-          <t>Moyen</t>
-        </is>
-      </c>
-      <c r="G99" s="73" t="n">
+      <c r="C100" s="71" t="inlineStr">
+        <is>
+          <t>Délibérations du Conseil d'Administration autorisant les placements et les ouvertures de comptes (DAT BOA, DAT Orabank, FCP géré par United Capital), comme l'exige l'article 85 des statuts.</t>
+        </is>
+      </c>
+      <c r="E100" s="72" t="inlineStr">
+        <is>
+          <t>Urgent</t>
+        </is>
+      </c>
+      <c r="G100" s="73" t="n">
         <v>46314</v>
       </c>
-      <c r="H99" s="73" t="n">
+      <c r="H100" s="73" t="n">
         <v>46321</v>
       </c>
-      <c r="I99" s="73" t="n"/>
-      <c r="J99" s="74" t="n"/>
-      <c r="K99" s="75" t="inlineStr">
+      <c r="I100" s="73" t="n"/>
+      <c r="J100" s="74" t="n"/>
+      <c r="K100" s="75" t="inlineStr">
         <is>
           <t>Demande issue de la lecture des statuts et du règlement intérieur du 15/06/2023 (PBC complémentaire textes et personnel).
-Fusion du 23/10/2026 : reprend l'ancien item 77 (« Convention collective et accord d'entreprise applicables au personnel du FPPN, articles fixant l'indemnité de départ à la retraite. »), statut « Non Reçu ».</t>
-        </is>
-      </c>
-      <c r="M99" s="76" t="inlineStr">
+Pointage des autres équipes (22/10/2026) : À rechercher dans les PV du CA reçus par l'équipe comptable (2020 et 2023 manquants).</t>
+        </is>
+      </c>
+      <c r="M100" s="76" t="inlineStr">
         <is>
           <t>Non Reçu</t>
         </is>
       </c>
     </row>
-    <row r="100" ht="18" customHeight="1" s="48">
-      <c r="C100" s="69" t="inlineStr">
-        <is>
-          <t>Décisions des organes (lecture des textes du 15/06/2023)</t>
-        </is>
-      </c>
-    </row>
-    <row r="101" ht="72" customHeight="1" s="48">
+    <row r="101" ht="132" customHeight="1" s="48">
       <c r="B101" s="70">
-        <f>+B99+1</f>
+        <f>+B100+1</f>
         <v/>
       </c>
       <c r="C101" s="71" t="inlineStr">
         <is>
-          <t>Délibérations du Conseil d'Administration autorisant les placements et les ouvertures de comptes (DAT BOA, DAT Orabank, FCP géré par United Capital), comme l'exige l'article 85 des statuts.</t>
+          <t>Délibération du Conseil d'Administration approuvant le cadre organique des emplois de la Direction Générale et la grille des salaires et indemnités (articles 61 et 66 des statuts).</t>
         </is>
       </c>
       <c r="E101" s="72" t="inlineStr">
         <is>
-          <t>Urgent</t>
+          <t>Faible</t>
         </is>
       </c>
       <c r="G101" s="73" t="n">
@@ -4142,73 +4143,72 @@
       <c r="H101" s="73" t="n">
         <v>46321</v>
       </c>
-      <c r="I101" s="73" t="n"/>
+      <c r="I101" s="73" t="n">
+        <v>46317</v>
+      </c>
       <c r="J101" s="74" t="n"/>
       <c r="K101" s="75" t="inlineStr">
         <is>
           <t>Demande issue de la lecture des statuts et du règlement intérieur du 15/06/2023 (PBC complémentaire textes et personnel).
-Pointage des autres équipes (22/10/2026) : À rechercher dans les PV du CA reçus par l'équipe comptable (2020 et 2023 manquants).</t>
+Pointage des autres équipes (22/10/2026) : À rechercher dans les PV du CA reçus par l'équipe comptable.
+Lu le 22/10/2026 : Organigrammes 2020 et 2021 reçus (« OrganigrammeFPPN_ORI (A) 2020.docx », « ORGANIGRAMME FPPN 2021(1).pdf », « COURRIER DE NOMINATION DÉFINITIVE.pdf ») ; délibération approuvant le cadre organique non reçue.</t>
         </is>
       </c>
       <c r="M101" s="76" t="inlineStr">
         <is>
-          <t>Non Reçu</t>
-        </is>
-      </c>
-    </row>
-    <row r="102" ht="132" customHeight="1" s="48">
-      <c r="B102" s="70">
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="18" customHeight="1" s="48">
+      <c r="C102" s="69" t="inlineStr">
+        <is>
+          <t>Documents reçus le 22/10/2026 (demandes complémentaires)</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="87" customHeight="1" s="48">
+      <c r="B103" s="70">
         <f>+B101+1</f>
         <v/>
       </c>
-      <c r="C102" s="71" t="inlineStr">
-        <is>
-          <t>Délibération du Conseil d'Administration approuvant le cadre organique des emplois de la Direction Générale et la grille des salaires et indemnités (articles 61 et 66 des statuts).</t>
-        </is>
-      </c>
-      <c r="E102" s="72" t="inlineStr">
-        <is>
-          <t>Faible</t>
-        </is>
-      </c>
-      <c r="G102" s="73" t="n">
-        <v>46314</v>
-      </c>
-      <c r="H102" s="73" t="n">
-        <v>46321</v>
-      </c>
-      <c r="I102" s="73" t="n">
+      <c r="C103" s="71" t="inlineStr">
+        <is>
+          <t>Version des comptes 2023 approuvée par l'Assemblée générale (les états financiers scannés portent un actif brut de 16 157 155 123 FCFA et un excédent de 928 699 102 FCFA, la balance et le rapport de gestion corrigé 16 167 155 123 FCFA et 930 629 102 FCFA) et explication de l'écart de résultat au 31/08/2026 (états financiers -437 148 460 FCFA, balance -441 256 500 FCFA).</t>
+        </is>
+      </c>
+      <c r="E103" s="72" t="inlineStr">
+        <is>
+          <t>Urgent</t>
+        </is>
+      </c>
+      <c r="G103" s="73" t="n">
         <v>46317</v>
       </c>
-      <c r="J102" s="74" t="n"/>
-      <c r="K102" s="75" t="inlineStr">
-        <is>
-          <t>Demande issue de la lecture des statuts et du règlement intérieur du 15/06/2023 (PBC complémentaire textes et personnel).
-Pointage des autres équipes (22/10/2026) : À rechercher dans les PV du CA reçus par l'équipe comptable.
-Lots 2 et 3 lus le 22/10/2026 : Organigrammes 2020 et 2021 reçus (« OrganigrammeFPPN_ORI (A) 2020.docx », « ORGANIGRAMME FPPN 2021(1).pdf », « COURRIER DE NOMINATION DÉFINITIVE.pdf ») ; délibération approuvant le cadre organique non reçue.</t>
-        </is>
-      </c>
-      <c r="M102" s="76" t="inlineStr">
-        <is>
-          <t>Partiellement Reçu</t>
-        </is>
-      </c>
-    </row>
-    <row r="103" ht="18" customHeight="1" s="48">
-      <c r="C103" s="69" t="inlineStr">
-        <is>
-          <t>Documents reçus le 22/10/2026 (demandes issues du rapport v9)</t>
-        </is>
-      </c>
-    </row>
-    <row r="104" ht="87" customHeight="1" s="48">
+      <c r="H103" s="73" t="n">
+        <v>46324</v>
+      </c>
+      <c r="I103" s="73" t="n"/>
+      <c r="J103" s="74" t="n"/>
+      <c r="K103" s="75" t="inlineStr">
+        <is>
+          <t>Demande issue des contrôles croisés du rapport (partie 3).</t>
+        </is>
+      </c>
+      <c r="M103" s="76" t="inlineStr">
+        <is>
+          <t>Non Reçu</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="75" customHeight="1" s="48">
       <c r="B104" s="70">
-        <f>+B102+1</f>
+        <f>+B103+1</f>
         <v/>
       </c>
       <c r="C104" s="71" t="inlineStr">
         <is>
-          <t>Version des comptes 2023 approuvée par l'Assemblée générale (les états financiers scannés portent un actif brut de 16 157 155 123 FCFA et un excédent de 928 699 102 FCFA, la balance et le rapport de gestion corrigé 16 167 155 123 FCFA et 930 629 102 FCFA) et explication de l'écart de résultat au 31/08/2026 (états financiers -437 148 460 FCFA, balance -441 256 500 FCFA).</t>
+          <t>Rapport de gestion 2025 rectifié présentant le solde de l'épargne due aux mutualistes au 31/12/2025 (PEP et EFC), distinct des cotisations collectées dans l'année (4 387 823 635 FCFA présentés comme l'épargne au 31/12/2025).</t>
         </is>
       </c>
       <c r="E104" s="72" t="inlineStr">
@@ -4226,7 +4226,7 @@
       <c r="J104" s="74" t="n"/>
       <c r="K104" s="75" t="inlineStr">
         <is>
-          <t>Demande issue des contrôles croisés du rapport v9 (partie 3).</t>
+          <t>Demande issue du rapport (partie 6).</t>
         </is>
       </c>
       <c r="M104" s="76" t="inlineStr">
@@ -4235,19 +4235,19 @@
         </is>
       </c>
     </row>
-    <row r="105" ht="75" customHeight="1" s="48">
+    <row r="105" ht="147" customHeight="1" s="48">
       <c r="B105" s="70">
         <f>+B104+1</f>
         <v/>
       </c>
       <c r="C105" s="71" t="inlineStr">
         <is>
-          <t>Clé de répartition maladie (936) / décès (8Z6) appliquée en janvier et février 2024 (rapport médian 8Z6 / 936 de 0,3059 et 0,3023, contre 0,3263 ensuite) et liste des dix adhérents d'écart entre l'étude des ratios et les fichiers 8Z6 de janvier à juin 2026.</t>
+          <t>Personnel : âge de départ à la retraite appliqué, nombre d'enfants à charge de chaque salarié, justification des douze dates d'embauche modifiées dans la DISA 2025, rattachement (Direction Générale, CMP, Grenier) des dix-neuf agents recrutés en 2025, note et fichiers de calcul de la provision pour départ à la retraite (compte 196) de 2020 à 2026 : méthode, hypothèses, liste des salariés.</t>
         </is>
       </c>
       <c r="E105" s="72" t="inlineStr">
         <is>
-          <t>Moyen</t>
+          <t>Urgent</t>
         </is>
       </c>
       <c r="G105" s="73" t="n">
@@ -4260,7 +4260,9 @@
       <c r="J105" s="74" t="n"/>
       <c r="K105" s="75" t="inlineStr">
         <is>
-          <t>Demande issue des contrôles croisés du rapport v9 (partie 3).</t>
+          <t>Demande issue du recalcul de la provision du personnel (rapport, partie 9).
+Fusion du 23/10/2026 : reprend l'ancien item 78 (« Note de calcul de la provision pour indemnités de départ à la retraite (compte 196) : méthode, hypothèses, liste des salariés. »), statut « Non Reçu ».
+Fusion du 23/10/2026 : reprend l'ancien item 98 (« Fichiers de calcul de la provision pour départ à la retraite de 2020 à 2026 (complète l'item 78). »), statut « Non Reçu ».</t>
         </is>
       </c>
       <c r="M105" s="76" t="inlineStr">
@@ -4269,48 +4271,21 @@
         </is>
       </c>
     </row>
-    <row r="106" ht="75" customHeight="1" s="48">
-      <c r="B106" s="70">
+    <row r="106" ht="18" customHeight="1" s="48">
+      <c r="C106" s="69" t="inlineStr">
+        <is>
+          <t>Dossier « 08-Nouveaux Dossiers Compta » reçu le 22/10/2026 (demandes issues de la revue actuarielle)</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="75" customHeight="1" s="48">
+      <c r="B107" s="70">
         <f>+B105+1</f>
         <v/>
       </c>
-      <c r="C106" s="71" t="inlineStr">
-        <is>
-          <t>Rapport de gestion 2025 rectifié présentant le solde de l'épargne due aux mutualistes au 31/12/2025 (PEP et EFC), distinct des cotisations collectées dans l'année (4 387 823 635 FCFA présentés comme l'épargne au 31/12/2025).</t>
-        </is>
-      </c>
-      <c r="E106" s="72" t="inlineStr">
-        <is>
-          <t>Urgent</t>
-        </is>
-      </c>
-      <c r="G106" s="73" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H106" s="73" t="n">
-        <v>46324</v>
-      </c>
-      <c r="I106" s="73" t="n"/>
-      <c r="J106" s="74" t="n"/>
-      <c r="K106" s="75" t="inlineStr">
-        <is>
-          <t>Demande issue du rapport v9 (partie 6).</t>
-        </is>
-      </c>
-      <c r="M106" s="76" t="inlineStr">
-        <is>
-          <t>Non Reçu</t>
-        </is>
-      </c>
-    </row>
-    <row r="107" ht="75" customHeight="1" s="48">
-      <c r="B107" s="70">
-        <f>+B106+1</f>
-        <v/>
-      </c>
       <c r="C107" s="71" t="inlineStr">
         <is>
-          <t>Personnel : âge de départ à la retraite appliqué, nombre d'enfants à charge de chaque salarié, justification des douze dates d'embauche modifiées dans la DISA 2025, rattachement (DG, CMP, Grenier) des dix-neuf agents recrutés en 2025, note de calcul du compte 196 (complète les items 78 et 98).</t>
+          <t>Liste des dossiers d'allocations décès composant le solde du compte 41591000 au 31/08/2026 (489 419 669 FCFA avec le compte 41592000) : nom, grade, date du décès, date de dépôt de la demande, montant, motif du non-paiement.</t>
         </is>
       </c>
       <c r="E107" s="72" t="inlineStr">
@@ -4328,7 +4303,7 @@
       <c r="J107" s="74" t="n"/>
       <c r="K107" s="75" t="inlineStr">
         <is>
-          <t>Demande issue du recalcul de la provision du personnel (rapport v9, partie 9).</t>
+          <t>Demande issue de la revue des provisions décès (rapport, partie 9).</t>
         </is>
       </c>
       <c r="M107" s="76" t="inlineStr">
@@ -4344,7 +4319,7 @@
       </c>
       <c r="C108" s="71" t="inlineStr">
         <is>
-          <t>Annexe 2 de la convention IPS-CGRAE (bulletin de souscription), barème de la cotisation des retraités et liste des retraités souscripteurs non précomptés faute de quotité cessible suffisante.</t>
+          <t>Texte qui fonde l'exclusion du suicide (quatre décès valorisés à 0 FCFA dans l'état 2025) et barème officiel 1 400 000, 1 600 000 et 2 200 000 FCFA appliqué dans les états.</t>
         </is>
       </c>
       <c r="E108" s="72" t="inlineStr">
@@ -4362,7 +4337,7 @@
       <c r="J108" s="74" t="n"/>
       <c r="K108" s="75" t="inlineStr">
         <is>
-          <t>Demande issue de la lecture de la convention IPS-CGRAE (rapport v9, partie 8).</t>
+          <t>Demande issue de la lecture des états de fin d'année des allocations décès.</t>
         </is>
       </c>
       <c r="M108" s="76" t="inlineStr">
@@ -4371,21 +4346,48 @@
         </is>
       </c>
     </row>
-    <row r="109" ht="18" customHeight="1" s="48">
-      <c r="C109" s="69" t="inlineStr">
-        <is>
-          <t>Dossier « 08-Nouveaux Dossiers Compta » reçu le 22/10/2026 (demandes issues de la revue actuarielle)</t>
+    <row r="109" ht="75" customHeight="1" s="48">
+      <c r="B109" s="70">
+        <f>+B108+1</f>
+        <v/>
+      </c>
+      <c r="C109" s="71" t="inlineStr">
+        <is>
+          <t>Décision de désignation ou de prolongation du directeur général après la mandature 2020-2023, et délégation de pouvoir pour les placements.</t>
+        </is>
+      </c>
+      <c r="E109" s="72" t="inlineStr">
+        <is>
+          <t>Urgent</t>
+        </is>
+      </c>
+      <c r="G109" s="73" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H109" s="73" t="n">
+        <v>46324</v>
+      </c>
+      <c r="I109" s="73" t="n"/>
+      <c r="J109" s="74" t="n"/>
+      <c r="K109" s="75" t="inlineStr">
+        <is>
+          <t>Demande issue de la lecture de l'attestation de désignation du 04/09/2020.</t>
+        </is>
+      </c>
+      <c r="M109" s="76" t="inlineStr">
+        <is>
+          <t>Non Reçu</t>
         </is>
       </c>
     </row>
     <row r="110" ht="75" customHeight="1" s="48">
       <c r="B110" s="70">
-        <f>+B108+1</f>
+        <f>+B109+1</f>
         <v/>
       </c>
       <c r="C110" s="71" t="inlineStr">
         <is>
-          <t>Liste des dossiers d'allocations décès composant le solde du compte 41591000 au 31/08/2026 (489 419 669 FCFA avec le compte 41592000) : nom, grade, date du décès, date de dépôt de la demande, montant, motif du non-paiement.</t>
+          <t>Projet de Cocody : budget, plan de financement, calendrier, décision des organes, rendement attendu, part financée par l'épargne.</t>
         </is>
       </c>
       <c r="E110" s="72" t="inlineStr">
@@ -4403,7 +4405,7 @@
       <c r="J110" s="74" t="n"/>
       <c r="K110" s="75" t="inlineStr">
         <is>
-          <t>Demande issue de la revue des provisions décès (rapport, partie 9).</t>
+          <t>Demande issue de la dérogation d'urbanisme de janvier 2025 (rapport, partie 9.3).</t>
         </is>
       </c>
       <c r="M110" s="76" t="inlineStr">
@@ -4412,14 +4414,14 @@
         </is>
       </c>
     </row>
-    <row r="111" ht="75" customHeight="1" s="48">
+    <row r="111" ht="87" customHeight="1" s="48">
       <c r="B111" s="70">
         <f>+B110+1</f>
         <v/>
       </c>
       <c r="C111" s="71" t="inlineStr">
         <is>
-          <t>Texte qui fonde l'exclusion du suicide (quatre décès valorisés à 0 FCFA dans l'état 2025) et barème officiel 1 400 000, 1 600 000 et 2 200 000 FCFA appliqué dans les états.</t>
+          <t>Comptabilité séparée du Centre médical du FPPN (CMP) et résultats annuels de 2020 à 2025.</t>
         </is>
       </c>
       <c r="E111" s="72" t="inlineStr">
@@ -4433,16 +4435,19 @@
       <c r="H111" s="73" t="n">
         <v>46324</v>
       </c>
-      <c r="I111" s="73" t="n"/>
+      <c r="I111" s="73" t="n">
+        <v>46317</v>
+      </c>
       <c r="J111" s="74" t="n"/>
       <c r="K111" s="75" t="inlineStr">
         <is>
-          <t>Demande issue de la lecture des états de fin d'année des allocations décès.</t>
+          <t>Demande issue de l'arrêté d'autorisation du CMP et du règlement d'exécution n° 004/2022, art. 27.
+Fusion du 23/10/2026 : reprend l'ancien item 88 (« Bilan d'ouverture de la clinique du FPPN (CMP) et détail des comptes 47111104 et 47111105. »), statut « Partiellement Reçu ».</t>
         </is>
       </c>
       <c r="M111" s="76" t="inlineStr">
         <is>
-          <t>Non Reçu</t>
+          <t>Partiellement Reçu</t>
         </is>
       </c>
     </row>
@@ -4453,12 +4458,12 @@
       </c>
       <c r="C112" s="71" t="inlineStr">
         <is>
-          <t>Décision de désignation ou de prolongation du directeur général après la mandature 2020-2023, et délégation de pouvoir pour les placements.</t>
+          <t>Fichiers de la CGRAE avec la date de naissance de tous les retraités (seuls les fichiers retour de février à avril 2024 la portent, pour 105 retraités) et prestations payées aux retraités.</t>
         </is>
       </c>
       <c r="E112" s="72" t="inlineStr">
         <is>
-          <t>Urgent</t>
+          <t>Moyen</t>
         </is>
       </c>
       <c r="G112" s="73" t="n">
@@ -4471,7 +4476,7 @@
       <c r="J112" s="74" t="n"/>
       <c r="K112" s="75" t="inlineStr">
         <is>
-          <t>Demande issue de la lecture de l'attestation de désignation du 04/09/2020.</t>
+          <t>Demande issue de la revue de la santé des retraités (rapport, partie 8).</t>
         </is>
       </c>
       <c r="M112" s="76" t="inlineStr">
@@ -4480,48 +4485,21 @@
         </is>
       </c>
     </row>
-    <row r="113" ht="75" customHeight="1" s="48">
-      <c r="B113" s="70">
+    <row r="113" s="48">
+      <c r="C113" s="69" t="inlineStr">
+        <is>
+          <t>Demandes issues de la vérification de cohérence du 23/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="57" customHeight="1" s="48">
+      <c r="B114" s="70">
         <f>+B112+1</f>
         <v/>
       </c>
-      <c r="C113" s="71" t="inlineStr">
-        <is>
-          <t>Projet de Cocody : budget, plan de financement, calendrier, décision des organes, rendement attendu, part financée par l'épargne.</t>
-        </is>
-      </c>
-      <c r="E113" s="72" t="inlineStr">
-        <is>
-          <t>Urgent</t>
-        </is>
-      </c>
-      <c r="G113" s="73" t="n">
-        <v>46317</v>
-      </c>
-      <c r="H113" s="73" t="n">
-        <v>46324</v>
-      </c>
-      <c r="I113" s="73" t="n"/>
-      <c r="J113" s="74" t="n"/>
-      <c r="K113" s="75" t="inlineStr">
-        <is>
-          <t>Demande issue de la dérogation d'urbanisme de janvier 2025 (rapport, partie 9.3).</t>
-        </is>
-      </c>
-      <c r="M113" s="76" t="inlineStr">
-        <is>
-          <t>Non Reçu</t>
-        </is>
-      </c>
-    </row>
-    <row r="114" ht="87" customHeight="1" s="48">
-      <c r="B114" s="70">
-        <f>+B113+1</f>
-        <v/>
-      </c>
       <c r="C114" s="71" t="inlineStr">
         <is>
-          <t>Comptabilité séparée du Centre médical du FPPN (CMP) et résultats annuels de 2020 à 2025.</t>
+          <t>Nature des références PTI, RPEP, EP, TI, R-PEP et PTQ précomptées au poste 998 de 2020 à août 2026 (174 461 860 FCFA à côté des références PEP) : remboursements de prêts PEP (comptes 27110000 et 27120000) ou autre produit.</t>
         </is>
       </c>
       <c r="E114" s="72" t="inlineStr">
@@ -4530,35 +4508,32 @@
         </is>
       </c>
       <c r="G114" s="73" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="H114" s="73" t="n">
-        <v>46324</v>
-      </c>
-      <c r="I114" s="73" t="n">
-        <v>46317</v>
-      </c>
+        <v>46325</v>
+      </c>
+      <c r="I114" s="73" t="n"/>
       <c r="J114" s="74" t="n"/>
       <c r="K114" s="75" t="inlineStr">
         <is>
-          <t>Demande issue de l'arrêté d'autorisation du CMP et du règlement d'exécution n° 004/2022, art. 27.
-Fusion du 23/10/2026 : reprend l'ancien item 88 (« Bilan d'ouverture de la clinique du FPPN (CMP) et détail des comptes 47111104 et 47111105. »), statut « Partiellement Reçu ».</t>
+          <t>Demande issue de la vérification de cohérence des chiffres du 23/10/2026.</t>
         </is>
       </c>
       <c r="M114" s="76" t="inlineStr">
         <is>
-          <t>Partiellement Reçu</t>
-        </is>
-      </c>
-    </row>
-    <row r="115" ht="75" customHeight="1" s="48">
+          <t>Non Reçu</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="57" customHeight="1" s="48">
       <c r="B115" s="70">
         <f>+B114+1</f>
         <v/>
       </c>
       <c r="C115" s="71" t="inlineStr">
         <is>
-          <t>Fichiers de la CGRAE avec la date de naissance de tous les retraités (seuls les fichiers retour de février à avril 2024 la portent, pour 105 retraités) et prestations payées aux retraités.</t>
+          <t>Explication de l'écart sur les sinistres décès 2021 : 156 020 000 FCFA dans « ETUDE DES RATIO MALADIE DECES 2.xlsx », contre 401 856 666 FCFA au compte 60210000 de la balance 2021.</t>
         </is>
       </c>
       <c r="E115" s="72" t="inlineStr">
@@ -4567,16 +4542,16 @@
         </is>
       </c>
       <c r="G115" s="73" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="H115" s="73" t="n">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="I115" s="73" t="n"/>
       <c r="J115" s="74" t="n"/>
       <c r="K115" s="75" t="inlineStr">
         <is>
-          <t>Demande issue de la revue de la santé des retraités (rapport, partie 8).</t>
+          <t>Demande issue de la vérification de cohérence des chiffres du 23/10/2026.</t>
         </is>
       </c>
       <c r="M115" s="76" t="inlineStr">
@@ -4585,26 +4560,53 @@
         </is>
       </c>
     </row>
-    <row r="116" s="48">
-      <c r="C116" s="69" t="inlineStr">
-        <is>
-          <t>Demandes issues de la vérification de cohérence du 23/10/2026</t>
+    <row r="116" ht="57" customHeight="1" s="48">
+      <c r="B116" s="70">
+        <f>+B115+1</f>
+        <v/>
+      </c>
+      <c r="C116" s="71" t="inlineStr">
+        <is>
+          <t>Validation, ligne par ligne, des montants décès supérieurs à 1 000 000 FCFA présents dans les fichiers retour 8Z6 (liste jointe par Adenka), et montant correct de chaque ligne.</t>
+        </is>
+      </c>
+      <c r="E116" s="72" t="inlineStr">
+        <is>
+          <t>Faible</t>
+        </is>
+      </c>
+      <c r="G116" s="73" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H116" s="73" t="n">
+        <v>46325</v>
+      </c>
+      <c r="I116" s="73" t="n"/>
+      <c r="J116" s="74" t="n"/>
+      <c r="K116" s="75" t="inlineStr">
+        <is>
+          <t>Demande issue de la vérification de cohérence des chiffres du 23/10/2026.</t>
+        </is>
+      </c>
+      <c r="M116" s="76" t="inlineStr">
+        <is>
+          <t>Non Reçu</t>
         </is>
       </c>
     </row>
     <row r="117" ht="57" customHeight="1" s="48">
       <c r="B117" s="70">
-        <f>+B115+1</f>
+        <f>+B116+1</f>
         <v/>
       </c>
       <c r="C117" s="71" t="inlineStr">
         <is>
-          <t>Nature des références PTI, RPEP, EP, TI, R-PEP et PTQ précomptées au poste 998 de 2020 à août 2026 (174 461 860 FCFA à côté des références PEP) : remboursements de prêts PEP (comptes 27110000 et 27120000) ou autre produit.</t>
+          <t>Procédure écrite du circuit des fichiers aller et retour de chaque produit (maladie, décès, EFC, PEP, Grenier, MEDOC, flotte, retraités) : qui produit, qui transmet, qui reçoit, qui rapproche.</t>
         </is>
       </c>
       <c r="E117" s="72" t="inlineStr">
         <is>
-          <t>Moyen</t>
+          <t>Faible</t>
         </is>
       </c>
       <c r="G117" s="73" t="n">
@@ -4626,14 +4628,14 @@
         </is>
       </c>
     </row>
-    <row r="118" ht="57" customHeight="1" s="48">
+    <row r="118" ht="42" customHeight="1" s="48">
       <c r="B118" s="70">
         <f>+B117+1</f>
         <v/>
       </c>
       <c r="C118" s="71" t="inlineStr">
         <is>
-          <t>Explication de l'écart sur les sinistres décès 2021 : 156 020 000 FCFA dans « ETUDE DES RATIO MALADIE DECES 2.xlsx », contre 401 856 666 FCFA au compte 60210000 de la balance 2021.</t>
+          <t>Effectif total de la Police nationale au 31/12 de 2020 à 2025 et au 31/08/2026 (taux de pénétration, Décision n° 05/2022).</t>
         </is>
       </c>
       <c r="E118" s="72" t="inlineStr">
@@ -4667,12 +4669,12 @@
       </c>
       <c r="C119" s="71" t="inlineStr">
         <is>
-          <t>Validation, ligne par ligne, des montants décès supérieurs à 1 000 000 FCFA présents dans les fichiers retour 8Z6 (liste jointe par Adenka), et montant correct de chaque ligne.</t>
+          <t>Grenier : explication de la hausse des retards de fin janvier 2026, et mode de règlement des échéances non précomptées par la Solde (paiement direct, compensation, relance).</t>
         </is>
       </c>
       <c r="E119" s="72" t="inlineStr">
         <is>
-          <t>Faible</t>
+          <t>Moyen</t>
         </is>
       </c>
       <c r="G119" s="73" t="n">
@@ -4694,108 +4696,9 @@
         </is>
       </c>
     </row>
-    <row r="120" ht="57" customHeight="1" s="48">
-      <c r="B120" s="70">
-        <f>+B119+1</f>
-        <v/>
-      </c>
-      <c r="C120" s="71" t="inlineStr">
-        <is>
-          <t>Procédure écrite du circuit des fichiers aller et retour de chaque produit (maladie, décès, EFC, PEP, Grenier, MEDOC, flotte, retraités) : qui produit, qui transmet, qui reçoit, qui rapproche.</t>
-        </is>
-      </c>
-      <c r="E120" s="72" t="inlineStr">
-        <is>
-          <t>Faible</t>
-        </is>
-      </c>
-      <c r="G120" s="73" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H120" s="73" t="n">
-        <v>46325</v>
-      </c>
-      <c r="I120" s="73" t="n"/>
-      <c r="J120" s="74" t="n"/>
-      <c r="K120" s="75" t="inlineStr">
-        <is>
-          <t>Demande issue de la vérification de cohérence des chiffres du 23/10/2026.</t>
-        </is>
-      </c>
-      <c r="M120" s="76" t="inlineStr">
-        <is>
-          <t>Non Reçu</t>
-        </is>
-      </c>
-    </row>
-    <row r="121" ht="42" customHeight="1" s="48">
-      <c r="B121" s="70">
-        <f>+B120+1</f>
-        <v/>
-      </c>
-      <c r="C121" s="71" t="inlineStr">
-        <is>
-          <t>Effectif total de la Police nationale au 31/12 de 2020 à 2025 et au 31/08/2026 (taux de pénétration, Décision n° 05/2022).</t>
-        </is>
-      </c>
-      <c r="E121" s="72" t="inlineStr">
-        <is>
-          <t>Moyen</t>
-        </is>
-      </c>
-      <c r="G121" s="73" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H121" s="73" t="n">
-        <v>46325</v>
-      </c>
-      <c r="I121" s="73" t="n"/>
-      <c r="J121" s="74" t="n"/>
-      <c r="K121" s="75" t="inlineStr">
-        <is>
-          <t>Demande issue de la vérification de cohérence des chiffres du 23/10/2026.</t>
-        </is>
-      </c>
-      <c r="M121" s="76" t="inlineStr">
-        <is>
-          <t>Non Reçu</t>
-        </is>
-      </c>
-    </row>
-    <row r="122" ht="57" customHeight="1" s="48">
-      <c r="B122" s="70">
-        <f>+B121+1</f>
-        <v/>
-      </c>
-      <c r="C122" s="71" t="inlineStr">
-        <is>
-          <t>Grenier : explication de la hausse des retards de fin janvier 2026, et mode de règlement des échéances non précomptées par la Solde (paiement direct, compensation, relance).</t>
-        </is>
-      </c>
-      <c r="E122" s="72" t="inlineStr">
-        <is>
-          <t>Moyen</t>
-        </is>
-      </c>
-      <c r="G122" s="73" t="n">
-        <v>46318</v>
-      </c>
-      <c r="H122" s="73" t="n">
-        <v>46325</v>
-      </c>
-      <c r="I122" s="73" t="n"/>
-      <c r="J122" s="74" t="n"/>
-      <c r="K122" s="75" t="inlineStr">
-        <is>
-          <t>Demande issue de la vérification de cohérence des chiffres du 23/10/2026.</t>
-        </is>
-      </c>
-      <c r="M122" s="76" t="inlineStr">
-        <is>
-          <t>Non Reçu</t>
-        </is>
-      </c>
-    </row>
+    <row r="120" s="48"/>
+    <row r="121" s="48"/>
+    <row r="122" s="48"/>
     <row r="123" s="48"/>
     <row r="124" s="48"/>
     <row r="125" s="48"/>
@@ -4874,7 +4777,7 @@
     <mergeCell ref="C5:M5"/>
     <mergeCell ref="C4:M4"/>
   </mergeCells>
-  <conditionalFormatting sqref="M11:M122">
+  <conditionalFormatting sqref="M11:M119">
     <cfRule type="cellIs" rank="0" priority="2" equalAverage="0" operator="equal" aboveAverage="0" dxfId="6" text="" percent="0" bottom="0">
       <formula>"Partiellement Reçu"</formula>
     </cfRule>
@@ -4885,7 +4788,7 @@
       <formula>"Reçu"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E11:E122">
+  <conditionalFormatting sqref="E11:E119">
     <cfRule type="cellIs" rank="0" priority="5" equalAverage="0" operator="equal" aboveAverage="0" dxfId="9" text="" percent="0" bottom="0">
       <formula>"Faible"</formula>
     </cfRule>
@@ -4897,13 +4800,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="E11:E122" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E11:E119" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Urgent,Moyen,Faible"</formula1>
     </dataValidation>
-    <dataValidation sqref="J11:J122" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J11:J119" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Physique,Electronique,Physique et Electronique"</formula1>
     </dataValidation>
-    <dataValidation sqref="M11:M122" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M11:M119" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Reçu,Non Reçu,Non Applicable,Partiellement Reçu"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4940,14 +4843,14 @@
     <row r="2">
       <c r="B2" s="97" t="inlineStr">
         <is>
-          <t>Pointage sur le contenu du lot 1 des nouveaux fichiers (22/10/2026)</t>
+          <t>Pointage sur le contenu des nouveaux fichiers (première partie) (22/10/2026)</t>
         </is>
       </c>
     </row>
     <row r="3" ht="40" customHeight="1" s="48">
       <c r="B3" s="79" t="inlineStr">
         <is>
-          <t>Lot 1 : 61 fichiers reçus, empreintes SHA-256 conformes au journal « journal_lot1.csv ». Chaque statut repose sur la lecture du contenu. Contrôle croisé : les nouvelles balances 2021 et 2025 sont identiques, compte par compte, aux balances déjà exploitées (aucun écart de solde).</t>
+          <t>61 fichiers reçus le 22/10/2026, contrôlés à réception. Chaque statut repose sur la lecture du contenu. Contrôle croisé : les nouvelles balances 2021 et 2025 sont identiques, compte par compte, aux balances déjà exploitées (aucun écart de solde).</t>
         </is>
       </c>
     </row>
@@ -5531,14 +5434,14 @@
     <row r="2">
       <c r="B2" s="97" t="inlineStr">
         <is>
-          <t>Pointage sur le contenu des lots 2 et 3 des nouveaux fichiers (22/10/2026)</t>
+          <t>Pointage sur le contenu des nouveaux fichiers (deuxième partie) (22/10/2026)</t>
         </is>
       </c>
     </row>
     <row r="3" ht="48" customHeight="1" s="48">
       <c r="B3" s="79" t="inlineStr">
         <is>
-          <t>Lot 2 : 26 fichiers, lot 3 : 29 fichiers, empreintes SHA-256 conformes aux journaux « journal_lot2.csv » et « journal_lot3.csv ». Les scans ont été lus par reconnaissance de caractères et les montants cités vérifiés sur l'image. Reçus sans item de la PBC : budgets de 2020 à 2026, PV d'arrêté de caisse de 2020 au 26/08/2026, convention DEPA. Items 110 à 114 ajoutés.</t>
+          <t>55 fichiers reçus le 22/10/2026, contrôlés à réception.csv » et « journal_lot3.csv ». Les scans ont été lus par reconnaissance de caractères et les montants cités vérifiés sur l'image. Reçus sans item de la PBC : budgets de 2020 à 2026, PV d'arrêté de caisse de 2020 au 26/08/2026, convention DEPA. Items 110 à 114 ajoutés.</t>
         </is>
       </c>
     </row>
@@ -5990,7 +5893,7 @@
       </c>
       <c r="F22" s="95" t="inlineStr">
         <is>
-          <t>Lot 3 : DISA et DASC 2021 à 2025 scannées et états des travailleurs occasionnels 2024 et 2025, en double des fichiers Excel du lot 1.</t>
+          <t>DISA et DASC 2021 à 2025 scannées et états des travailleurs occasionnels 2024 et 2025, en double des fichiers Excel reçus.</t>
         </is>
       </c>
     </row>
@@ -6115,7 +6018,7 @@
       </c>
       <c r="F27" s="95" t="inlineStr">
         <is>
-          <t>Demande issue des contrôles croisés du rapport v9 (partie 3).</t>
+          <t>Demande issue des contrôles croisés du rapport (partie 3).</t>
         </is>
       </c>
     </row>
@@ -6140,7 +6043,7 @@
       </c>
       <c r="F28" s="95" t="inlineStr">
         <is>
-          <t>Demande issue des contrôles croisés du rapport v9 (partie 3).</t>
+          <t>Demande issue des contrôles croisés du rapport (partie 3).</t>
         </is>
       </c>
     </row>
@@ -6165,7 +6068,7 @@
       </c>
       <c r="F29" s="95" t="inlineStr">
         <is>
-          <t>Demande issue du rapport v9 (partie 6).</t>
+          <t>Demande issue du rapport (partie 6).</t>
         </is>
       </c>
     </row>
@@ -6190,7 +6093,7 @@
       </c>
       <c r="F30" s="95" t="inlineStr">
         <is>
-          <t>Demande issue du recalcul de la provision du personnel (rapport v9, partie 9).</t>
+          <t>Demande issue du recalcul de la provision du personnel (rapport, partie 9).</t>
         </is>
       </c>
     </row>
@@ -6215,7 +6118,7 @@
       </c>
       <c r="F31" s="95" t="inlineStr">
         <is>
-          <t>Demande issue de la lecture de la convention IPS-CGRAE (rapport v9, partie 8).</t>
+          <t>Demande issue de la lecture de la convention IPS-CGRAE (rapport, partie 8).</t>
         </is>
       </c>
     </row>
@@ -6682,7 +6585,7 @@
         <v>2</v>
       </c>
       <c r="B7" s="101" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C7" s="103" t="inlineStr">
         <is>
@@ -6864,7 +6767,7 @@
         <v>16</v>
       </c>
       <c r="B21" s="101" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C21" s="103" t="inlineStr">
         <is>
@@ -6890,7 +6793,7 @@
         <v>18</v>
       </c>
       <c r="B23" s="101" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C23" s="103" t="inlineStr">
         <is>
@@ -6916,7 +6819,7 @@
         <v>20</v>
       </c>
       <c r="B25" s="101" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C25" s="103" t="inlineStr">
         <is>
@@ -7072,7 +6975,7 @@
         <v>32</v>
       </c>
       <c r="B37" s="101" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C37" s="103" t="inlineStr">
         <is>
@@ -7085,7 +6988,7 @@
         <v>33</v>
       </c>
       <c r="B38" s="101" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C38" s="103" t="inlineStr">
         <is>
@@ -7137,7 +7040,7 @@
         <v>37</v>
       </c>
       <c r="B42" s="101" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C42" s="103" t="inlineStr">
         <is>
@@ -7254,7 +7157,7 @@
         <v>46</v>
       </c>
       <c r="B51" s="101" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C51" s="103" t="inlineStr">
         <is>
@@ -7306,7 +7209,7 @@
         <v>50</v>
       </c>
       <c r="B55" s="101" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C55" s="103" t="inlineStr">
         <is>
@@ -7540,7 +7443,7 @@
         <v>68</v>
       </c>
       <c r="B73" s="101" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C73" s="103" t="inlineStr">
         <is>
@@ -7644,7 +7547,7 @@
         <v>76</v>
       </c>
       <c r="B81" s="101" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C81" s="103" t="inlineStr">
         <is>
@@ -7657,7 +7560,7 @@
         <v>77</v>
       </c>
       <c r="B82" s="101" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C82" s="103" t="inlineStr">
         <is>
@@ -7670,11 +7573,11 @@
         <v>78</v>
       </c>
       <c r="B83" s="101" t="n">
-        <v>52</v>
-      </c>
-      <c r="C83" s="102" t="inlineStr">
-        <is>
-          <t>Conservé</t>
+        <v>78</v>
+      </c>
+      <c r="C83" s="103" t="inlineStr">
+        <is>
+          <t>Fusionné avec l'ancien item 113 (doublon)</t>
         </is>
       </c>
     </row>
@@ -7683,7 +7586,7 @@
         <v>79</v>
       </c>
       <c r="B84" s="101" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C84" s="102" t="inlineStr">
         <is>
@@ -7696,7 +7599,7 @@
         <v>80</v>
       </c>
       <c r="B85" s="101" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C85" s="102" t="inlineStr">
         <is>
@@ -7709,7 +7612,7 @@
         <v>81</v>
       </c>
       <c r="B86" s="101" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C86" s="102" t="inlineStr">
         <is>
@@ -7722,7 +7625,7 @@
         <v>82</v>
       </c>
       <c r="B87" s="101" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C87" s="102" t="inlineStr">
         <is>
@@ -7735,7 +7638,7 @@
         <v>83</v>
       </c>
       <c r="B88" s="101" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C88" s="102" t="inlineStr">
         <is>
@@ -7748,7 +7651,7 @@
         <v>84</v>
       </c>
       <c r="B89" s="101" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C89" s="102" t="inlineStr">
         <is>
@@ -7761,7 +7664,7 @@
         <v>85</v>
       </c>
       <c r="B90" s="101" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C90" s="102" t="inlineStr">
         <is>
@@ -7774,7 +7677,7 @@
         <v>86</v>
       </c>
       <c r="B91" s="101" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C91" s="102" t="inlineStr">
         <is>
@@ -7787,7 +7690,7 @@
         <v>87</v>
       </c>
       <c r="B92" s="101" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C92" s="102" t="inlineStr">
         <is>
@@ -7800,7 +7703,7 @@
         <v>88</v>
       </c>
       <c r="B93" s="101" t="n">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C93" s="103" t="inlineStr">
         <is>
@@ -7813,7 +7716,7 @@
         <v>89</v>
       </c>
       <c r="B94" s="101" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C94" s="102" t="inlineStr">
         <is>
@@ -7826,7 +7729,7 @@
         <v>90</v>
       </c>
       <c r="B95" s="101" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C95" s="102" t="inlineStr">
         <is>
@@ -7839,7 +7742,7 @@
         <v>91</v>
       </c>
       <c r="B96" s="101" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C96" s="102" t="inlineStr">
         <is>
@@ -7852,7 +7755,7 @@
         <v>92</v>
       </c>
       <c r="B97" s="101" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C97" s="102" t="inlineStr">
         <is>
@@ -7878,7 +7781,7 @@
         <v>94</v>
       </c>
       <c r="B99" s="101" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C99" s="102" t="inlineStr">
         <is>
@@ -7891,7 +7794,7 @@
         <v>95</v>
       </c>
       <c r="B100" s="101" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C100" s="102" t="inlineStr">
         <is>
@@ -7904,7 +7807,7 @@
         <v>96</v>
       </c>
       <c r="B101" s="101" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C101" s="102" t="inlineStr">
         <is>
@@ -7917,7 +7820,7 @@
         <v>97</v>
       </c>
       <c r="B102" s="101" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C102" s="102" t="inlineStr">
         <is>
@@ -7930,11 +7833,11 @@
         <v>98</v>
       </c>
       <c r="B103" s="101" t="n">
-        <v>52</v>
+        <v>78</v>
       </c>
       <c r="C103" s="103" t="inlineStr">
         <is>
-          <t>Fusionné avec l'ancien item 78 (doublon)</t>
+          <t>Fusionné avec l'ancien item 113 (doublon)</t>
         </is>
       </c>
     </row>
@@ -7943,7 +7846,7 @@
         <v>99</v>
       </c>
       <c r="B104" s="101" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C104" s="102" t="inlineStr">
         <is>
@@ -7956,7 +7859,7 @@
         <v>100</v>
       </c>
       <c r="B105" s="101" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C105" s="102" t="inlineStr">
         <is>
@@ -7982,7 +7885,7 @@
         <v>102</v>
       </c>
       <c r="B107" s="101" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C107" s="102" t="inlineStr">
         <is>
@@ -7995,7 +7898,7 @@
         <v>103</v>
       </c>
       <c r="B108" s="101" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C108" s="102" t="inlineStr">
         <is>
@@ -8008,7 +7911,7 @@
         <v>104</v>
       </c>
       <c r="B109" s="101" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C109" s="102" t="inlineStr">
         <is>
@@ -8021,7 +7924,7 @@
         <v>105</v>
       </c>
       <c r="B110" s="101" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C110" s="102" t="inlineStr">
         <is>
@@ -8060,7 +7963,7 @@
         <v>108</v>
       </c>
       <c r="B113" s="101" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C113" s="103" t="inlineStr">
         <is>
@@ -8073,7 +7976,7 @@
         <v>109</v>
       </c>
       <c r="B114" s="101" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C114" s="102" t="inlineStr">
         <is>
@@ -8086,7 +7989,7 @@
         <v>110</v>
       </c>
       <c r="B115" s="101" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C115" s="102" t="inlineStr">
         <is>
@@ -8099,11 +8002,11 @@
         <v>111</v>
       </c>
       <c r="B116" s="101" t="n">
-        <v>78</v>
-      </c>
-      <c r="C116" s="102" t="inlineStr">
-        <is>
-          <t>Conservé</t>
+        <v>34</v>
+      </c>
+      <c r="C116" s="103" t="inlineStr">
+        <is>
+          <t>Fusionné avec l'ancien item 56 (doublon)</t>
         </is>
       </c>
     </row>
@@ -8112,7 +8015,7 @@
         <v>112</v>
       </c>
       <c r="B117" s="101" t="n">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C117" s="102" t="inlineStr">
         <is>
@@ -8125,7 +8028,7 @@
         <v>113</v>
       </c>
       <c r="B118" s="101" t="n">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C118" s="102" t="inlineStr">
         <is>
@@ -8138,11 +8041,11 @@
         <v>114</v>
       </c>
       <c r="B119" s="101" t="n">
-        <v>81</v>
-      </c>
-      <c r="C119" s="102" t="inlineStr">
-        <is>
-          <t>Conservé</t>
+        <v>2</v>
+      </c>
+      <c r="C119" s="103" t="inlineStr">
+        <is>
+          <t>Fusionné avec l'ancien item 4 (doublon)</t>
         </is>
       </c>
     </row>
@@ -8151,7 +8054,7 @@
         <v>115</v>
       </c>
       <c r="B120" s="101" t="n">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C120" s="102" t="inlineStr">
         <is>
@@ -8164,7 +8067,7 @@
         <v>116</v>
       </c>
       <c r="B121" s="101" t="n">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C121" s="102" t="inlineStr">
         <is>
@@ -8177,7 +8080,7 @@
         <v>117</v>
       </c>
       <c r="B122" s="101" t="n">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C122" s="102" t="inlineStr">
         <is>
@@ -8190,7 +8093,7 @@
         <v>118</v>
       </c>
       <c r="B123" s="101" t="n">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C123" s="102" t="inlineStr">
         <is>
@@ -8203,7 +8106,7 @@
         <v>119</v>
       </c>
       <c r="B124" s="101" t="n">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C124" s="102" t="inlineStr">
         <is>
@@ -8216,7 +8119,7 @@
         <v>120</v>
       </c>
       <c r="B125" s="101" t="n">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C125" s="102" t="inlineStr">
         <is>
@@ -8297,12 +8200,12 @@
         </is>
       </c>
       <c r="C6" s="95">
-        <f>COUNTIF('PBC Actuariat FPPN'!$M$11:$M$122,"Reçu")</f>
+        <f>COUNTIF('PBC Actuariat FPPN'!$M$11:$M$119,"Reçu")</f>
         <v/>
       </c>
       <c r="D6" s="95" t="inlineStr">
         <is>
-          <t>33, 46, 50, 63, 71, 72</t>
+          <t>33, 46, 50, 62, 70, 71</t>
         </is>
       </c>
     </row>
@@ -8313,12 +8216,12 @@
         </is>
       </c>
       <c r="C7" s="95">
-        <f>COUNTIF('PBC Actuariat FPPN'!$M$11:$M$122,"Partiellement Reçu")</f>
+        <f>COUNTIF('PBC Actuariat FPPN'!$M$11:$M$119,"Partiellement Reçu")</f>
         <v/>
       </c>
       <c r="D7" s="95" t="inlineStr">
         <is>
-          <t>1, 2, 3, 4, 6, 7, 9, 10, 12, 14, 15, 16, 17, 19, 20, 25, 27, 28, 31, 34, 35, 47, 48, 49, 53, 54, 56, 57, 58, 59, 60, 62, 64, 65, 69, 70, 73, 76, 86</t>
+          <t>1, 2, 3, 4, 6, 7, 9, 10, 12, 14, 15, 16, 17, 19, 20, 25, 27, 28, 31, 34, 35, 47, 48, 49, 52, 53, 55, 56, 57, 58, 59, 61, 63, 64, 68, 69, 72, 75, 83</t>
         </is>
       </c>
     </row>
@@ -8329,12 +8232,12 @@
         </is>
       </c>
       <c r="C8" s="95">
-        <f>COUNTIF('PBC Actuariat FPPN'!$M$11:$M$122,"Non Reçu")</f>
+        <f>COUNTIF('PBC Actuariat FPPN'!$M$11:$M$119,"Non Reçu")</f>
         <v/>
       </c>
       <c r="D8" s="95" t="inlineStr">
         <is>
-          <t>5, 8, 11, 13, 18, 21, 22, 23, 24, 26, 29, 30, 32, 36, 37, 38, 39, 40, 41, 42, 43, 44, 45, 51, 52, 55, 61, 66, 67, 68, 74, 75, 77, 78, 79, 80, 81, 82, 83, 84, 85, 87, 88, 89, 90, 91, 92, 93</t>
+          <t>5, 8, 11, 13, 18, 21, 22, 23, 24, 26, 29, 30, 32, 36, 37, 38, 39, 40, 41, 42, 43, 44, 45, 51, 54, 60, 65, 66, 67, 73, 74, 76, 77, 78, 79, 80, 81, 82, 84, 85, 86, 87, 88, 89, 90</t>
         </is>
       </c>
     </row>
@@ -8350,7 +8253,7 @@
       </c>
       <c r="D9" s="95" t="inlineStr">
         <is>
-          <t>1 à 93</t>
+          <t>1 à 90</t>
         </is>
       </c>
     </row>
@@ -11380,7 +11283,7 @@
         </is>
       </c>
       <c r="C18" s="87" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D18" s="88" t="inlineStr">
         <is>

</xml_diff>